<commit_message>
changes from Friday. progress table and synapsida marg rates issue
</commit_message>
<xml_diff>
--- a/analyses_log.xlsx
+++ b/analyses_log.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Git\BDNN_Arielli\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\SimoesLabAdmin\Documents\BDNN_Arielli\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{F99CE426-57FB-4A01-9014-693AA1AEC635}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0637504D-DCFF-4624-AA26-9E5E0B2FB6FE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-103" yWindow="-103" windowWidth="33120" windowHeight="18000" xr2:uid="{2B31D40A-C581-4DA9-854D-6A8F263900C8}"/>
+    <workbookView xWindow="840" yWindow="729" windowWidth="23091" windowHeight="16020" xr2:uid="{2B31D40A-C581-4DA9-854D-6A8F263900C8}"/>
   </bookViews>
   <sheets>
     <sheet name="table" sheetId="2" r:id="rId1"/>
@@ -1430,8 +1430,8 @@
       <c r="M15" s="3" t="s">
         <v>33</v>
       </c>
-      <c r="N15" s="4" t="s">
-        <v>15</v>
+      <c r="N15" s="3" t="s">
+        <v>14</v>
       </c>
       <c r="O15" s="4" t="s">
         <v>15</v>
@@ -1816,8 +1816,8 @@
       <c r="M22" s="3" t="s">
         <v>33</v>
       </c>
-      <c r="N22" s="4" t="s">
-        <v>15</v>
+      <c r="N22" s="3" t="s">
+        <v>14</v>
       </c>
       <c r="O22" s="4" t="s">
         <v>15</v>

</xml_diff>

<commit_message>
pulled B_bdnn restored for tem from cluster, update to progress log
</commit_message>
<xml_diff>
--- a/analyses_log.xlsx
+++ b/analyses_log.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\SimoesLabAdmin\Documents\BDNN_Arielli\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0637504D-DCFF-4624-AA26-9E5E0B2FB6FE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F59A9633-B5F2-4EE8-BEC8-147D7A0F082B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="840" yWindow="729" windowWidth="23091" windowHeight="16020" xr2:uid="{2B31D40A-C581-4DA9-854D-6A8F263900C8}"/>
+    <workbookView xWindow="-189" yWindow="934" windowWidth="23092" windowHeight="16020" xr2:uid="{2B31D40A-C581-4DA9-854D-6A8F263900C8}"/>
   </bookViews>
   <sheets>
     <sheet name="table" sheetId="2" r:id="rId1"/>
@@ -1109,8 +1109,8 @@
       <c r="N9" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="O9" s="4" t="s">
-        <v>15</v>
+      <c r="O9" s="3" t="s">
+        <v>14</v>
       </c>
       <c r="P9" s="3" t="s">
         <v>12</v>
@@ -1165,8 +1165,8 @@
       <c r="N10" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="O10" s="4" t="s">
-        <v>15</v>
+      <c r="O10" s="3" t="s">
+        <v>14</v>
       </c>
       <c r="P10" s="3" t="s">
         <v>12</v>

</xml_diff>

<commit_message>
A_mcmc scripts, B_covar renamed to B_covar_rjmcmc, edits to progress log
</commit_message>
<xml_diff>
--- a/analyses_log.xlsx
+++ b/analyses_log.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\SimoesLabAdmin\Documents\BDNN_Arielli\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F59A9633-B5F2-4EE8-BEC8-147D7A0F082B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C382C5C8-3587-4D4B-8609-1A33F850F2A9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-189" yWindow="934" windowWidth="23092" windowHeight="16020" xr2:uid="{2B31D40A-C581-4DA9-854D-6A8F263900C8}"/>
+    <workbookView xWindow="283" yWindow="1774" windowWidth="27111" windowHeight="16020" xr2:uid="{2B31D40A-C581-4DA9-854D-6A8F263900C8}"/>
   </bookViews>
   <sheets>
     <sheet name="table" sheetId="2" r:id="rId1"/>
@@ -47,7 +47,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="346" uniqueCount="58">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="352" uniqueCount="62">
   <si>
     <t>Sampling Algorithm</t>
   </si>
@@ -221,6 +221,18 @@
   </si>
   <si>
     <t>Age Sampling Replicates</t>
+  </si>
+  <si>
+    <t>MCMC</t>
+  </si>
+  <si>
+    <t>Compare with 1 Myr RJMCMC, no preds</t>
+  </si>
+  <si>
+    <t>Compare with 1 Myr BDMCMC, no preds, and CoVar RJMCMC</t>
+  </si>
+  <si>
+    <t>CoVa + MBD</t>
   </si>
 </sst>
 </file>
@@ -673,7 +685,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A9EA881A-93D2-4F0C-B578-B509C4BBF0BD}">
-  <dimension ref="A1:S22"/>
+  <dimension ref="A1:S24"/>
   <sheetFormatPr defaultRowHeight="12.9" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="1" max="1" width="18.3046875" style="7" customWidth="1"/>
@@ -692,7 +704,7 @@
     <col min="15" max="15" width="13.07421875" style="3" bestFit="1" customWidth="1"/>
     <col min="16" max="16" width="12.84375" style="3" bestFit="1" customWidth="1"/>
     <col min="17" max="17" width="13.07421875" style="3" customWidth="1"/>
-    <col min="18" max="18" width="35.3046875" style="3" customWidth="1"/>
+    <col min="18" max="18" width="48.15234375" style="3" customWidth="1"/>
     <col min="19" max="16384" width="9.23046875" style="3"/>
   </cols>
   <sheetData>
@@ -752,38 +764,72 @@
         <v>24</v>
       </c>
     </row>
-    <row r="2" spans="1:19" s="9" customFormat="1" x14ac:dyDescent="0.4">
-      <c r="A2" s="9" t="s">
+    <row r="2" spans="1:19" s="2" customFormat="1" x14ac:dyDescent="0.4">
+      <c r="A2" s="7" t="s">
         <v>17</v>
       </c>
-      <c r="B2" s="10" t="s">
-        <v>32</v>
-      </c>
-      <c r="C2" s="9" t="s">
+      <c r="B2" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="C2" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="D2" s="9" t="s">
+      <c r="D2" s="3" t="s">
         <v>48</v>
       </c>
-      <c r="E2" s="9" t="s">
-        <v>40</v>
-      </c>
-      <c r="F2" s="9" t="s">
-        <v>40</v>
-      </c>
-      <c r="G2" s="9" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="3" spans="1:19" s="2" customFormat="1" x14ac:dyDescent="0.4">
+      <c r="E2" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="F2" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="G2" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="H2" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="I2" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="J2" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="K2" s="3">
+        <v>10</v>
+      </c>
+      <c r="L2" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="M2" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="N2" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="O2" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="P2" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="Q2" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="R2" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="S2" s="3"/>
+    </row>
+    <row r="3" spans="1:19" x14ac:dyDescent="0.4">
       <c r="A3" s="7" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B3" s="1" t="s">
         <v>31</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="D3" s="3" t="s">
         <v>48</v>
@@ -827,213 +873,130 @@
       <c r="Q3" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="R3" s="3"/>
-      <c r="S3" s="3"/>
-    </row>
-    <row r="4" spans="1:19" x14ac:dyDescent="0.4">
-      <c r="A4" s="7" t="s">
+      <c r="R3" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="S3" s="2"/>
+    </row>
+    <row r="4" spans="1:19" s="9" customFormat="1" x14ac:dyDescent="0.4">
+      <c r="B4" s="10" t="s">
+        <v>32</v>
+      </c>
+      <c r="C4" s="9" t="s">
+        <v>58</v>
+      </c>
+      <c r="D4" s="9" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="5" spans="1:19" s="9" customFormat="1" x14ac:dyDescent="0.4">
+      <c r="B5" s="10" t="s">
+        <v>31</v>
+      </c>
+      <c r="C5" s="9" t="s">
+        <v>58</v>
+      </c>
+      <c r="D5" s="9" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="6" spans="1:19" x14ac:dyDescent="0.4">
+      <c r="A6" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="C6" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="B4" s="1" t="s">
+      <c r="D6" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="E6" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="F6" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="G6" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="H6" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="I6" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="J6" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="K6" s="3">
+        <v>10</v>
+      </c>
+      <c r="L6" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="M6" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="N6" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="O6" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="P6" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="Q6" s="3" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="7" spans="1:19" s="9" customFormat="1" x14ac:dyDescent="0.4">
+      <c r="B7" s="10" t="s">
         <v>31</v>
       </c>
-      <c r="C4" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="D4" s="3" t="s">
-        <v>48</v>
-      </c>
-      <c r="E4" s="3" t="s">
-        <v>40</v>
-      </c>
-      <c r="F4" s="3" t="s">
-        <v>40</v>
-      </c>
-      <c r="G4" s="3" t="s">
-        <v>40</v>
-      </c>
-      <c r="H4" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="I4" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="J4" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="K4" s="3">
-        <v>10</v>
-      </c>
-      <c r="L4" s="3" t="s">
-        <v>34</v>
-      </c>
-      <c r="M4" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="N4" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="O4" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="P4" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="Q4" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="S4" s="2"/>
-    </row>
-    <row r="5" spans="1:19" x14ac:dyDescent="0.4">
-      <c r="A5" s="7" t="s">
-        <v>21</v>
-      </c>
-      <c r="B5" s="1" t="s">
-        <v>31</v>
-      </c>
-      <c r="C5" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="D5" s="3" t="s">
+      <c r="C7" s="9" t="s">
+        <v>58</v>
+      </c>
+      <c r="D7" s="9" t="s">
         <v>18</v>
       </c>
-      <c r="E5" s="3" t="s">
-        <v>40</v>
-      </c>
-      <c r="F5" s="3" t="s">
+      <c r="E7" s="9" t="s">
+        <v>40</v>
+      </c>
+      <c r="F7" s="9" t="s">
         <v>20</v>
       </c>
-      <c r="G5" s="3" t="s">
-        <v>40</v>
-      </c>
-      <c r="H5" s="3" t="s">
-        <v>40</v>
-      </c>
-      <c r="I5" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="J5" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="K5" s="3">
-        <v>10</v>
-      </c>
-      <c r="L5" s="3" t="s">
-        <v>34</v>
-      </c>
-      <c r="M5" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="N5" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="O5" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="P5" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="Q5" s="3" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="6" spans="1:19" s="9" customFormat="1" x14ac:dyDescent="0.4">
-      <c r="B6" s="10" t="s">
-        <v>31</v>
-      </c>
-      <c r="C6" s="9" t="s">
-        <v>17</v>
-      </c>
-      <c r="D6" s="9" t="s">
-        <v>18</v>
-      </c>
-      <c r="E6" s="9" t="s">
-        <v>40</v>
-      </c>
-      <c r="F6" s="9" t="s">
-        <v>20</v>
-      </c>
-      <c r="G6" s="9" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="7" spans="1:19" x14ac:dyDescent="0.4">
-      <c r="A7" s="7" t="s">
-        <v>18</v>
-      </c>
-      <c r="B7" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="C7" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="D7" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="E7" s="3" t="s">
-        <v>40</v>
-      </c>
-      <c r="F7" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="G7" s="3" t="s">
-        <v>40</v>
-      </c>
-      <c r="H7" s="3" t="s">
-        <v>40</v>
-      </c>
-      <c r="I7" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="J7" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="K7" s="3">
-        <v>10</v>
-      </c>
-      <c r="L7" s="3" t="s">
-        <v>34</v>
-      </c>
-      <c r="M7" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="N7" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="O7" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="P7" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="Q7" s="3" t="s">
-        <v>15</v>
+      <c r="G7" s="9" t="s">
+        <v>40</v>
       </c>
     </row>
     <row r="8" spans="1:19" x14ac:dyDescent="0.4">
       <c r="A8" s="7" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B8" s="1" t="s">
         <v>32</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>17</v>
+        <v>58</v>
       </c>
       <c r="D8" s="3" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E8" s="3" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="F8" s="3" t="s">
-        <v>27</v>
+        <v>20</v>
       </c>
       <c r="G8" s="3" t="s">
-        <v>51</v>
+        <v>40</v>
       </c>
       <c r="H8" s="3" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="I8" s="3" t="s">
         <v>11</v>
@@ -1041,8 +1004,8 @@
       <c r="J8" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="K8" s="3" t="s">
-        <v>56</v>
+      <c r="K8" s="3">
+        <v>10</v>
       </c>
       <c r="L8" s="3" t="s">
         <v>34</v>
@@ -1060,10 +1023,7 @@
         <v>12</v>
       </c>
       <c r="Q8" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="R8" s="3" t="s">
-        <v>29</v>
+        <v>15</v>
       </c>
     </row>
     <row r="9" spans="1:19" x14ac:dyDescent="0.4">
@@ -1074,13 +1034,13 @@
         <v>32</v>
       </c>
       <c r="C9" s="3" t="s">
-        <v>17</v>
+        <v>58</v>
       </c>
       <c r="D9" s="3" t="s">
         <v>19</v>
       </c>
       <c r="E9" s="3" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="F9" s="3" t="s">
         <v>27</v>
@@ -1116,7 +1076,7 @@
         <v>12</v>
       </c>
       <c r="Q9" s="3" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="R9" s="3" t="s">
         <v>29</v>
@@ -1130,13 +1090,13 @@
         <v>32</v>
       </c>
       <c r="C10" s="3" t="s">
-        <v>17</v>
+        <v>58</v>
       </c>
       <c r="D10" s="3" t="s">
         <v>19</v>
       </c>
       <c r="E10" s="3" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="F10" s="3" t="s">
         <v>27</v>
@@ -1180,25 +1140,25 @@
     </row>
     <row r="11" spans="1:19" x14ac:dyDescent="0.4">
       <c r="A11" s="7" t="s">
-        <v>9</v>
+        <v>19</v>
       </c>
       <c r="B11" s="1" t="s">
         <v>32</v>
       </c>
       <c r="C11" s="3" t="s">
-        <v>17</v>
+        <v>58</v>
       </c>
       <c r="D11" s="3" t="s">
-        <v>9</v>
+        <v>19</v>
       </c>
       <c r="E11" s="3" t="s">
-        <v>40</v>
-      </c>
-      <c r="F11" s="8" t="s">
-        <v>47</v>
-      </c>
-      <c r="G11" s="8" t="s">
-        <v>40</v>
+        <v>43</v>
+      </c>
+      <c r="F11" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="G11" s="3" t="s">
+        <v>51</v>
       </c>
       <c r="H11" s="3" t="s">
         <v>39</v>
@@ -1209,8 +1169,8 @@
       <c r="J11" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="K11" s="3">
-        <v>10</v>
+      <c r="K11" s="3" t="s">
+        <v>56</v>
       </c>
       <c r="L11" s="3" t="s">
         <v>34</v>
@@ -1230,58 +1190,25 @@
       <c r="Q11" s="3" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="12" spans="1:19" x14ac:dyDescent="0.4">
-      <c r="A12" s="7" t="s">
-        <v>9</v>
-      </c>
-      <c r="B12" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="C12" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="D12" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="E12" s="3" t="s">
-        <v>40</v>
-      </c>
-      <c r="F12" s="3" t="s">
-        <v>53</v>
-      </c>
-      <c r="G12" s="3" t="s">
-        <v>51</v>
-      </c>
-      <c r="H12" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="I12" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="J12" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="K12" s="3">
-        <v>10</v>
-      </c>
-      <c r="L12" s="3" t="s">
-        <v>34</v>
-      </c>
-      <c r="M12" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="N12" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="O12" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="P12" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="Q12" s="3" t="s">
-        <v>15</v>
+      <c r="R11" s="3" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="12" spans="1:19" s="9" customFormat="1" x14ac:dyDescent="0.4">
+      <c r="A12" s="9" t="s">
+        <v>61</v>
+      </c>
+      <c r="B12" s="10" t="s">
+        <v>31</v>
+      </c>
+      <c r="C12" s="9" t="s">
+        <v>58</v>
+      </c>
+      <c r="D12" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="E12" s="9" t="s">
+        <v>42</v>
       </c>
     </row>
     <row r="13" spans="1:19" x14ac:dyDescent="0.4">
@@ -1292,7 +1219,7 @@
         <v>32</v>
       </c>
       <c r="C13" s="3" t="s">
-        <v>17</v>
+        <v>58</v>
       </c>
       <c r="D13" s="3" t="s">
         <v>9</v>
@@ -1300,14 +1227,14 @@
       <c r="E13" s="3" t="s">
         <v>40</v>
       </c>
-      <c r="F13" s="3" t="s">
-        <v>53</v>
-      </c>
-      <c r="G13" s="3" t="s">
-        <v>51</v>
+      <c r="F13" s="8" t="s">
+        <v>47</v>
+      </c>
+      <c r="G13" s="8" t="s">
+        <v>40</v>
       </c>
       <c r="H13" s="3" t="s">
-        <v>28</v>
+        <v>39</v>
       </c>
       <c r="I13" s="3" t="s">
         <v>11</v>
@@ -1345,7 +1272,7 @@
         <v>32</v>
       </c>
       <c r="C14" s="3" t="s">
-        <v>17</v>
+        <v>58</v>
       </c>
       <c r="D14" s="3" t="s">
         <v>9</v>
@@ -1360,7 +1287,7 @@
         <v>51</v>
       </c>
       <c r="H14" s="3" t="s">
-        <v>26</v>
+        <v>37</v>
       </c>
       <c r="I14" s="3" t="s">
         <v>11</v>
@@ -1398,7 +1325,7 @@
         <v>32</v>
       </c>
       <c r="C15" s="3" t="s">
-        <v>17</v>
+        <v>58</v>
       </c>
       <c r="D15" s="3" t="s">
         <v>9</v>
@@ -1407,13 +1334,13 @@
         <v>40</v>
       </c>
       <c r="F15" s="3" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="G15" s="3" t="s">
-        <v>40</v>
+        <v>51</v>
       </c>
       <c r="H15" s="3" t="s">
-        <v>40</v>
+        <v>28</v>
       </c>
       <c r="I15" s="3" t="s">
         <v>11</v>
@@ -1433,8 +1360,8 @@
       <c r="N15" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="O15" s="4" t="s">
-        <v>15</v>
+      <c r="O15" s="3" t="s">
+        <v>14</v>
       </c>
       <c r="P15" s="3" t="s">
         <v>12</v>
@@ -1451,7 +1378,7 @@
         <v>32</v>
       </c>
       <c r="C16" s="3" t="s">
-        <v>17</v>
+        <v>58</v>
       </c>
       <c r="D16" s="3" t="s">
         <v>9</v>
@@ -1460,13 +1387,13 @@
         <v>40</v>
       </c>
       <c r="F16" s="3" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="G16" s="3" t="s">
-        <v>40</v>
+        <v>51</v>
       </c>
       <c r="H16" s="3" t="s">
-        <v>10</v>
+        <v>26</v>
       </c>
       <c r="I16" s="3" t="s">
         <v>11</v>
@@ -1501,10 +1428,10 @@
         <v>9</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="C17" s="3" t="s">
-        <v>17</v>
+        <v>58</v>
       </c>
       <c r="D17" s="3" t="s">
         <v>9</v>
@@ -1513,13 +1440,13 @@
         <v>40</v>
       </c>
       <c r="F17" s="3" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="G17" s="3" t="s">
         <v>40</v>
       </c>
       <c r="H17" s="3" t="s">
-        <v>10</v>
+        <v>40</v>
       </c>
       <c r="I17" s="3" t="s">
         <v>11</v>
@@ -1539,8 +1466,8 @@
       <c r="N17" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="O17" s="3" t="s">
-        <v>14</v>
+      <c r="O17" s="4" t="s">
+        <v>15</v>
       </c>
       <c r="P17" s="3" t="s">
         <v>12</v>
@@ -1548,19 +1475,16 @@
       <c r="Q17" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="R17" s="3" t="s">
-        <v>25</v>
-      </c>
     </row>
     <row r="18" spans="1:18" x14ac:dyDescent="0.4">
       <c r="A18" s="7" t="s">
         <v>9</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="C18" s="3" t="s">
-        <v>17</v>
+        <v>58</v>
       </c>
       <c r="D18" s="3" t="s">
         <v>9</v>
@@ -1569,13 +1493,13 @@
         <v>40</v>
       </c>
       <c r="F18" s="3" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="G18" s="3" t="s">
-        <v>52</v>
+        <v>40</v>
       </c>
       <c r="H18" s="3" t="s">
-        <v>35</v>
+        <v>10</v>
       </c>
       <c r="I18" s="3" t="s">
         <v>11</v>
@@ -1595,8 +1519,8 @@
       <c r="N18" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="O18" s="4" t="s">
-        <v>22</v>
+      <c r="O18" s="3" t="s">
+        <v>14</v>
       </c>
       <c r="P18" s="3" t="s">
         <v>12</v>
@@ -1604,9 +1528,6 @@
       <c r="Q18" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="R18" s="3" t="s">
-        <v>25</v>
-      </c>
     </row>
     <row r="19" spans="1:18" x14ac:dyDescent="0.4">
       <c r="A19" s="7" t="s">
@@ -1616,7 +1537,7 @@
         <v>31</v>
       </c>
       <c r="C19" s="3" t="s">
-        <v>17</v>
+        <v>58</v>
       </c>
       <c r="D19" s="3" t="s">
         <v>9</v>
@@ -1625,13 +1546,13 @@
         <v>40</v>
       </c>
       <c r="F19" s="3" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="G19" s="3" t="s">
-        <v>52</v>
+        <v>40</v>
       </c>
       <c r="H19" s="3" t="s">
-        <v>36</v>
+        <v>10</v>
       </c>
       <c r="I19" s="3" t="s">
         <v>11</v>
@@ -1651,8 +1572,8 @@
       <c r="N19" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="O19" s="4" t="s">
-        <v>22</v>
+      <c r="O19" s="3" t="s">
+        <v>14</v>
       </c>
       <c r="P19" s="3" t="s">
         <v>12</v>
@@ -1672,7 +1593,7 @@
         <v>31</v>
       </c>
       <c r="C20" s="3" t="s">
-        <v>17</v>
+        <v>58</v>
       </c>
       <c r="D20" s="3" t="s">
         <v>9</v>
@@ -1687,7 +1608,7 @@
         <v>52</v>
       </c>
       <c r="H20" s="3" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="I20" s="3" t="s">
         <v>11</v>
@@ -1728,7 +1649,7 @@
         <v>31</v>
       </c>
       <c r="C21" s="3" t="s">
-        <v>17</v>
+        <v>58</v>
       </c>
       <c r="D21" s="3" t="s">
         <v>9</v>
@@ -1743,7 +1664,7 @@
         <v>52</v>
       </c>
       <c r="H21" s="3" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="I21" s="3" t="s">
         <v>11</v>
@@ -1784,7 +1705,7 @@
         <v>31</v>
       </c>
       <c r="C22" s="3" t="s">
-        <v>17</v>
+        <v>58</v>
       </c>
       <c r="D22" s="3" t="s">
         <v>9</v>
@@ -1793,13 +1714,13 @@
         <v>40</v>
       </c>
       <c r="F22" s="3" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="G22" s="3" t="s">
-        <v>40</v>
+        <v>52</v>
       </c>
       <c r="H22" s="3" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="I22" s="3" t="s">
         <v>11</v>
@@ -1820,12 +1741,124 @@
         <v>14</v>
       </c>
       <c r="O22" s="4" t="s">
-        <v>15</v>
+        <v>22</v>
       </c>
       <c r="P22" s="3" t="s">
         <v>12</v>
       </c>
       <c r="Q22" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="R22" s="3" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="23" spans="1:18" x14ac:dyDescent="0.4">
+      <c r="A23" s="7" t="s">
+        <v>9</v>
+      </c>
+      <c r="B23" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="C23" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="D23" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="E23" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="F23" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="G23" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="H23" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="I23" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="J23" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="K23" s="3">
+        <v>10</v>
+      </c>
+      <c r="L23" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="M23" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="N23" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="O23" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="P23" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="Q23" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="R23" s="3" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="24" spans="1:18" x14ac:dyDescent="0.4">
+      <c r="A24" s="7" t="s">
+        <v>9</v>
+      </c>
+      <c r="B24" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="C24" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="D24" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="E24" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="F24" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="G24" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="H24" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="I24" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="J24" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="K24" s="3">
+        <v>10</v>
+      </c>
+      <c r="L24" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="M24" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="N24" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="O24" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="P24" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="Q24" s="3" t="s">
         <v>15</v>
       </c>
     </row>

</xml_diff>

<commit_message>
EOD tuesday progress log
</commit_message>
<xml_diff>
--- a/analyses_log.xlsx
+++ b/analyses_log.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\SimoesLabAdmin\Documents\BDNN_Arielli\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{762B8CCA-5D07-485E-87D7-222F722066B9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6DF6D6CF-CEEC-43C3-8510-59C3B3ECF2F8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="283" yWindow="1774" windowWidth="27111" windowHeight="16020" xr2:uid="{2B31D40A-C581-4DA9-854D-6A8F263900C8}"/>
   </bookViews>
@@ -47,7 +47,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="372" uniqueCount="64">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="389" uniqueCount="66">
   <si>
     <t>Sampling Algorithm</t>
   </si>
@@ -190,9 +190,6 @@
     <t>Original</t>
   </si>
   <si>
-    <t>?</t>
-  </si>
-  <si>
     <t>no predictor</t>
   </si>
   <si>
@@ -217,9 +214,6 @@
     <t>Time + Diversity</t>
   </si>
   <si>
-    <t>9*</t>
-  </si>
-  <si>
     <t>Age Sampling Replicates</t>
   </si>
   <si>
@@ -239,6 +233,18 @@
   </si>
   <si>
     <t>102 mi</t>
+  </si>
+  <si>
+    <t>103 mi</t>
+  </si>
+  <si>
+    <t>104 mi</t>
+  </si>
+  <si>
+    <t>105 mi</t>
+  </si>
+  <si>
+    <t>106 mi</t>
   </si>
 </sst>
 </file>
@@ -275,7 +281,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -291,12 +297,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="0"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFF99"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -336,11 +336,8 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
@@ -355,6 +352,9 @@
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
   </cellXfs>
@@ -731,7 +731,7 @@
         <v>0</v>
       </c>
       <c r="D1" s="5" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="E1" s="5" t="s">
         <v>45</v>
@@ -740,7 +740,7 @@
         <v>1</v>
       </c>
       <c r="G1" s="5" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="H1" s="5" t="s">
         <v>44</v>
@@ -752,7 +752,7 @@
         <v>3</v>
       </c>
       <c r="K1" s="5" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="L1" s="5" t="s">
         <v>4</v>
@@ -787,7 +787,7 @@
         <v>17</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="E2" s="3" t="s">
         <v>40</v>
@@ -829,7 +829,7 @@
         <v>14</v>
       </c>
       <c r="R2" s="3" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="S2" s="3"/>
     </row>
@@ -844,7 +844,7 @@
         <v>16</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="E3" s="3" t="s">
         <v>40</v>
@@ -886,19 +886,19 @@
         <v>14</v>
       </c>
       <c r="R3" s="3" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="S3" s="2"/>
     </row>
     <row r="4" spans="1:19" s="2" customFormat="1" x14ac:dyDescent="0.4">
-      <c r="B4" s="11" t="s">
+      <c r="B4" s="10" t="s">
         <v>32</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="E4" s="2" t="s">
         <v>40</v>
@@ -922,7 +922,7 @@
         <v>11</v>
       </c>
       <c r="L4" s="2" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="M4" s="2" t="s">
         <v>33</v>
@@ -930,19 +930,25 @@
       <c r="N4" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="O4" s="12" t="s">
+      <c r="O4" s="11" t="s">
+        <v>15</v>
+      </c>
+      <c r="P4" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="Q4" s="2" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="5" spans="1:19" s="2" customFormat="1" x14ac:dyDescent="0.4">
-      <c r="B5" s="11" t="s">
+      <c r="B5" s="10" t="s">
         <v>31</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="E5" s="3" t="s">
         <v>40</v>
@@ -966,7 +972,7 @@
         <v>12</v>
       </c>
       <c r="L5" s="3" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="M5" s="3" t="s">
         <v>33</v>
@@ -974,7 +980,13 @@
       <c r="N5" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="O5" s="12" t="s">
+      <c r="O5" s="11" t="s">
+        <v>15</v>
+      </c>
+      <c r="P5" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="Q5" s="2" t="s">
         <v>15</v>
       </c>
     </row>
@@ -1031,24 +1043,48 @@
         <v>14</v>
       </c>
     </row>
-    <row r="7" spans="1:19" s="9" customFormat="1" x14ac:dyDescent="0.4">
-      <c r="B7" s="10" t="s">
+    <row r="7" spans="1:19" s="8" customFormat="1" x14ac:dyDescent="0.4">
+      <c r="B7" s="9" t="s">
         <v>31</v>
       </c>
-      <c r="C7" s="9" t="s">
-        <v>58</v>
-      </c>
-      <c r="D7" s="9" t="s">
+      <c r="C7" s="8" t="s">
+        <v>56</v>
+      </c>
+      <c r="D7" s="8" t="s">
         <v>18</v>
       </c>
-      <c r="E7" s="9" t="s">
-        <v>40</v>
-      </c>
-      <c r="F7" s="9" t="s">
+      <c r="E7" s="8" t="s">
+        <v>40</v>
+      </c>
+      <c r="F7" s="8" t="s">
         <v>20</v>
       </c>
-      <c r="G7" s="9" t="s">
-        <v>40</v>
+      <c r="G7" s="8" t="s">
+        <v>40</v>
+      </c>
+      <c r="I7" s="8" t="s">
+        <v>11</v>
+      </c>
+      <c r="J7" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="K7" s="8">
+        <v>11</v>
+      </c>
+      <c r="L7" s="8" t="s">
+        <v>60</v>
+      </c>
+      <c r="M7" s="8" t="s">
+        <v>33</v>
+      </c>
+      <c r="N7" s="12" t="s">
+        <v>15</v>
+      </c>
+      <c r="P7" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="Q7" s="8" t="s">
+        <v>15</v>
       </c>
     </row>
     <row r="8" spans="1:19" x14ac:dyDescent="0.4">
@@ -1059,7 +1095,7 @@
         <v>32</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="D8" s="3" t="s">
         <v>18</v>
@@ -1083,10 +1119,10 @@
         <v>13</v>
       </c>
       <c r="K8" s="3">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="L8" s="3" t="s">
-        <v>34</v>
+        <v>61</v>
       </c>
       <c r="M8" s="3" t="s">
         <v>33</v>
@@ -1112,7 +1148,7 @@
         <v>32</v>
       </c>
       <c r="C9" s="3" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="D9" s="3" t="s">
         <v>19</v>
@@ -1124,7 +1160,7 @@
         <v>27</v>
       </c>
       <c r="G9" s="3" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="H9" s="3" t="s">
         <v>39</v>
@@ -1135,11 +1171,11 @@
       <c r="J9" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="K9" s="3" t="s">
-        <v>56</v>
+      <c r="K9" s="3">
+        <v>13</v>
       </c>
       <c r="L9" s="3" t="s">
-        <v>34</v>
+        <v>62</v>
       </c>
       <c r="M9" s="3" t="s">
         <v>33</v>
@@ -1168,7 +1204,7 @@
         <v>32</v>
       </c>
       <c r="C10" s="3" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="D10" s="3" t="s">
         <v>19</v>
@@ -1180,7 +1216,7 @@
         <v>27</v>
       </c>
       <c r="G10" s="3" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="H10" s="3" t="s">
         <v>39</v>
@@ -1191,11 +1227,11 @@
       <c r="J10" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="K10" s="3" t="s">
-        <v>56</v>
+      <c r="K10" s="3">
+        <v>14</v>
       </c>
       <c r="L10" s="3" t="s">
-        <v>34</v>
+        <v>63</v>
       </c>
       <c r="M10" s="3" t="s">
         <v>33</v>
@@ -1224,7 +1260,7 @@
         <v>32</v>
       </c>
       <c r="C11" s="3" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="D11" s="3" t="s">
         <v>19</v>
@@ -1236,7 +1272,7 @@
         <v>27</v>
       </c>
       <c r="G11" s="3" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="H11" s="3" t="s">
         <v>39</v>
@@ -1247,11 +1283,11 @@
       <c r="J11" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="K11" s="3" t="s">
-        <v>56</v>
+      <c r="K11" s="3">
+        <v>15</v>
       </c>
       <c r="L11" s="3" t="s">
-        <v>34</v>
+        <v>64</v>
       </c>
       <c r="M11" s="3" t="s">
         <v>33</v>
@@ -1272,21 +1308,51 @@
         <v>29</v>
       </c>
     </row>
-    <row r="12" spans="1:19" s="9" customFormat="1" x14ac:dyDescent="0.4">
-      <c r="A12" s="9" t="s">
-        <v>61</v>
-      </c>
-      <c r="B12" s="10" t="s">
+    <row r="12" spans="1:19" s="8" customFormat="1" x14ac:dyDescent="0.4">
+      <c r="A12" s="8" t="s">
+        <v>59</v>
+      </c>
+      <c r="B12" s="9" t="s">
         <v>31</v>
       </c>
-      <c r="C12" s="9" t="s">
-        <v>58</v>
-      </c>
-      <c r="D12" s="9" t="s">
+      <c r="C12" s="8" t="s">
+        <v>56</v>
+      </c>
+      <c r="D12" s="8" t="s">
         <v>19</v>
       </c>
-      <c r="E12" s="9" t="s">
+      <c r="E12" s="8" t="s">
         <v>42</v>
+      </c>
+      <c r="F12" s="8" t="s">
+        <v>27</v>
+      </c>
+      <c r="G12" s="8" t="s">
+        <v>50</v>
+      </c>
+      <c r="I12" s="8" t="s">
+        <v>11</v>
+      </c>
+      <c r="J12" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="K12" s="8">
+        <v>16</v>
+      </c>
+      <c r="L12" s="8" t="s">
+        <v>65</v>
+      </c>
+      <c r="M12" s="8" t="s">
+        <v>33</v>
+      </c>
+      <c r="N12" s="12" t="s">
+        <v>15</v>
+      </c>
+      <c r="P12" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="Q12" s="8" t="s">
+        <v>15</v>
       </c>
     </row>
     <row r="13" spans="1:19" x14ac:dyDescent="0.4">
@@ -1297,7 +1363,7 @@
         <v>32</v>
       </c>
       <c r="C13" s="3" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="D13" s="3" t="s">
         <v>9</v>
@@ -1305,11 +1371,11 @@
       <c r="E13" s="3" t="s">
         <v>40</v>
       </c>
-      <c r="F13" s="8" t="s">
-        <v>47</v>
-      </c>
-      <c r="G13" s="8" t="s">
-        <v>40</v>
+      <c r="F13" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="G13" s="3" t="s">
+        <v>50</v>
       </c>
       <c r="H13" s="3" t="s">
         <v>39</v>
@@ -1350,7 +1416,7 @@
         <v>32</v>
       </c>
       <c r="C14" s="3" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="D14" s="3" t="s">
         <v>9</v>
@@ -1359,10 +1425,10 @@
         <v>40</v>
       </c>
       <c r="F14" s="3" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="G14" s="3" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="H14" s="3" t="s">
         <v>37</v>
@@ -1403,7 +1469,7 @@
         <v>32</v>
       </c>
       <c r="C15" s="3" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="D15" s="3" t="s">
         <v>9</v>
@@ -1412,10 +1478,10 @@
         <v>40</v>
       </c>
       <c r="F15" s="3" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="G15" s="3" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="H15" s="3" t="s">
         <v>28</v>
@@ -1456,7 +1522,7 @@
         <v>32</v>
       </c>
       <c r="C16" s="3" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="D16" s="3" t="s">
         <v>9</v>
@@ -1465,10 +1531,10 @@
         <v>40</v>
       </c>
       <c r="F16" s="3" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="G16" s="3" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="H16" s="3" t="s">
         <v>26</v>
@@ -1509,7 +1575,7 @@
         <v>32</v>
       </c>
       <c r="C17" s="3" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="D17" s="3" t="s">
         <v>9</v>
@@ -1518,7 +1584,7 @@
         <v>40</v>
       </c>
       <c r="F17" s="3" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="G17" s="3" t="s">
         <v>40</v>
@@ -1562,7 +1628,7 @@
         <v>32</v>
       </c>
       <c r="C18" s="3" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="D18" s="3" t="s">
         <v>9</v>
@@ -1571,7 +1637,7 @@
         <v>40</v>
       </c>
       <c r="F18" s="3" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="G18" s="3" t="s">
         <v>40</v>
@@ -1615,7 +1681,7 @@
         <v>31</v>
       </c>
       <c r="C19" s="3" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="D19" s="3" t="s">
         <v>9</v>
@@ -1624,7 +1690,7 @@
         <v>40</v>
       </c>
       <c r="F19" s="3" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="G19" s="3" t="s">
         <v>40</v>
@@ -1671,7 +1737,7 @@
         <v>31</v>
       </c>
       <c r="C20" s="3" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="D20" s="3" t="s">
         <v>9</v>
@@ -1680,10 +1746,10 @@
         <v>40</v>
       </c>
       <c r="F20" s="3" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="G20" s="3" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="H20" s="3" t="s">
         <v>35</v>
@@ -1727,7 +1793,7 @@
         <v>31</v>
       </c>
       <c r="C21" s="3" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="D21" s="3" t="s">
         <v>9</v>
@@ -1736,10 +1802,10 @@
         <v>40</v>
       </c>
       <c r="F21" s="3" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="G21" s="3" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="H21" s="3" t="s">
         <v>36</v>
@@ -1783,7 +1849,7 @@
         <v>31</v>
       </c>
       <c r="C22" s="3" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="D22" s="3" t="s">
         <v>9</v>
@@ -1792,10 +1858,10 @@
         <v>40</v>
       </c>
       <c r="F22" s="3" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="G22" s="3" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="H22" s="3" t="s">
         <v>37</v>
@@ -1839,7 +1905,7 @@
         <v>31</v>
       </c>
       <c r="C23" s="3" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="D23" s="3" t="s">
         <v>9</v>
@@ -1848,10 +1914,10 @@
         <v>40</v>
       </c>
       <c r="F23" s="3" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="G23" s="3" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="H23" s="3" t="s">
         <v>38</v>
@@ -1895,7 +1961,7 @@
         <v>31</v>
       </c>
       <c r="C24" s="3" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="D24" s="3" t="s">
         <v>9</v>
@@ -1904,7 +1970,7 @@
         <v>40</v>
       </c>
       <c r="F24" s="3" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="G24" s="3" t="s">
         <v>40</v>

</xml_diff>

<commit_message>
B_covar_mcmc scripts, update to log reflecting that
</commit_message>
<xml_diff>
--- a/analyses_log.xlsx
+++ b/analyses_log.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\SimoesLabAdmin\Documents\BDNN_Arielli\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6DF6D6CF-CEEC-43C3-8510-59C3B3ECF2F8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9F39E905-2B73-4FFA-81A1-BF51CC1378AF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="283" yWindow="1774" windowWidth="27111" windowHeight="16020" xr2:uid="{2B31D40A-C581-4DA9-854D-6A8F263900C8}"/>
+    <workbookView xWindow="1543" yWindow="1311" windowWidth="27111" windowHeight="16020" xr2:uid="{2B31D40A-C581-4DA9-854D-6A8F263900C8}"/>
   </bookViews>
   <sheets>
     <sheet name="table" sheetId="2" r:id="rId1"/>
@@ -47,7 +47,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="389" uniqueCount="66">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="405" uniqueCount="59">
   <si>
     <t>Sampling Algorithm</t>
   </si>
@@ -224,27 +224,6 @@
   </si>
   <si>
     <t>Compare with 1 Myr BDMCMC, no preds, and CoVar RJMCMC</t>
-  </si>
-  <si>
-    <t>CoVa + MBD</t>
-  </si>
-  <si>
-    <t>101 mi</t>
-  </si>
-  <si>
-    <t>102 mi</t>
-  </si>
-  <si>
-    <t>103 mi</t>
-  </si>
-  <si>
-    <t>104 mi</t>
-  </si>
-  <si>
-    <t>105 mi</t>
-  </si>
-  <si>
-    <t>106 mi</t>
   </si>
 </sst>
 </file>
@@ -697,7 +676,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A9EA881A-93D2-4F0C-B578-B509C4BBF0BD}">
-  <dimension ref="A1:S24"/>
+  <dimension ref="A1:S25"/>
   <sheetFormatPr defaultRowHeight="12.9" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="1" max="1" width="18.3046875" style="7" customWidth="1"/>
@@ -918,11 +897,11 @@
       <c r="J4" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="K4" s="2">
-        <v>11</v>
-      </c>
-      <c r="L4" s="2" t="s">
-        <v>60</v>
+      <c r="K4" s="3">
+        <v>10</v>
+      </c>
+      <c r="L4" s="3" t="s">
+        <v>34</v>
       </c>
       <c r="M4" s="2" t="s">
         <v>33</v>
@@ -969,10 +948,10 @@
         <v>13</v>
       </c>
       <c r="K5" s="3">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="L5" s="3" t="s">
-        <v>61</v>
+        <v>34</v>
       </c>
       <c r="M5" s="3" t="s">
         <v>33</v>
@@ -1043,47 +1022,53 @@
         <v>14</v>
       </c>
     </row>
-    <row r="7" spans="1:19" s="8" customFormat="1" x14ac:dyDescent="0.4">
-      <c r="B7" s="9" t="s">
+    <row r="7" spans="1:19" s="2" customFormat="1" x14ac:dyDescent="0.4">
+      <c r="A7" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="B7" s="10" t="s">
         <v>31</v>
       </c>
-      <c r="C7" s="8" t="s">
+      <c r="C7" s="2" t="s">
         <v>56</v>
       </c>
-      <c r="D7" s="8" t="s">
+      <c r="D7" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="E7" s="8" t="s">
-        <v>40</v>
-      </c>
-      <c r="F7" s="8" t="s">
+      <c r="E7" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="F7" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="G7" s="8" t="s">
-        <v>40</v>
-      </c>
-      <c r="I7" s="8" t="s">
-        <v>11</v>
-      </c>
-      <c r="J7" s="8" t="s">
-        <v>13</v>
-      </c>
-      <c r="K7" s="8">
-        <v>11</v>
-      </c>
-      <c r="L7" s="8" t="s">
-        <v>60</v>
-      </c>
-      <c r="M7" s="8" t="s">
-        <v>33</v>
-      </c>
-      <c r="N7" s="12" t="s">
-        <v>15</v>
-      </c>
-      <c r="P7" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="Q7" s="8" t="s">
+      <c r="G7" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="I7" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="J7" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="K7" s="2">
+        <v>10</v>
+      </c>
+      <c r="L7" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="M7" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="N7" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="O7" s="11" t="s">
+        <v>15</v>
+      </c>
+      <c r="P7" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="Q7" s="2" t="s">
         <v>15</v>
       </c>
     </row>
@@ -1119,10 +1104,10 @@
         <v>13</v>
       </c>
       <c r="K8" s="3">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="L8" s="3" t="s">
-        <v>61</v>
+        <v>34</v>
       </c>
       <c r="M8" s="3" t="s">
         <v>33</v>
@@ -1172,10 +1157,10 @@
         <v>13</v>
       </c>
       <c r="K9" s="3">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="L9" s="3" t="s">
-        <v>62</v>
+        <v>34</v>
       </c>
       <c r="M9" s="3" t="s">
         <v>33</v>
@@ -1228,10 +1213,10 @@
         <v>13</v>
       </c>
       <c r="K10" s="3">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="L10" s="3" t="s">
-        <v>63</v>
+        <v>34</v>
       </c>
       <c r="M10" s="3" t="s">
         <v>33</v>
@@ -1284,10 +1269,10 @@
         <v>13</v>
       </c>
       <c r="K11" s="3">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="L11" s="3" t="s">
-        <v>64</v>
+        <v>34</v>
       </c>
       <c r="M11" s="3" t="s">
         <v>33</v>
@@ -1310,7 +1295,7 @@
     </row>
     <row r="12" spans="1:19" s="8" customFormat="1" x14ac:dyDescent="0.4">
       <c r="A12" s="8" t="s">
-        <v>59</v>
+        <v>19</v>
       </c>
       <c r="B12" s="9" t="s">
         <v>31</v>
@@ -1337,10 +1322,10 @@
         <v>13</v>
       </c>
       <c r="K12" s="8">
-        <v>16</v>
+        <v>10</v>
       </c>
       <c r="L12" s="8" t="s">
-        <v>65</v>
+        <v>34</v>
       </c>
       <c r="M12" s="8" t="s">
         <v>33</v>
@@ -1355,56 +1340,50 @@
         <v>15</v>
       </c>
     </row>
-    <row r="13" spans="1:19" x14ac:dyDescent="0.4">
-      <c r="A13" s="7" t="s">
-        <v>9</v>
-      </c>
-      <c r="B13" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="C13" s="3" t="s">
+    <row r="13" spans="1:19" s="8" customFormat="1" x14ac:dyDescent="0.4">
+      <c r="A13" s="8" t="s">
+        <v>19</v>
+      </c>
+      <c r="B13" s="9" t="s">
+        <v>31</v>
+      </c>
+      <c r="C13" s="8" t="s">
         <v>56</v>
       </c>
-      <c r="D13" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="E13" s="3" t="s">
-        <v>40</v>
-      </c>
-      <c r="F13" s="3" t="s">
-        <v>52</v>
-      </c>
-      <c r="G13" s="3" t="s">
+      <c r="D13" s="8" t="s">
+        <v>19</v>
+      </c>
+      <c r="E13" s="8" t="s">
+        <v>43</v>
+      </c>
+      <c r="F13" s="8" t="s">
+        <v>27</v>
+      </c>
+      <c r="G13" s="8" t="s">
         <v>50</v>
       </c>
-      <c r="H13" s="3" t="s">
-        <v>39</v>
-      </c>
-      <c r="I13" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="J13" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="K13" s="3">
-        <v>10</v>
-      </c>
-      <c r="L13" s="3" t="s">
-        <v>34</v>
-      </c>
-      <c r="M13" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="N13" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="O13" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="P13" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="Q13" s="3" t="s">
+      <c r="I13" s="8" t="s">
+        <v>11</v>
+      </c>
+      <c r="J13" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="K13" s="8">
+        <v>10</v>
+      </c>
+      <c r="L13" s="8" t="s">
+        <v>34</v>
+      </c>
+      <c r="M13" s="8" t="s">
+        <v>33</v>
+      </c>
+      <c r="N13" s="12" t="s">
+        <v>15</v>
+      </c>
+      <c r="P13" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="Q13" s="8" t="s">
         <v>15</v>
       </c>
     </row>
@@ -1431,7 +1410,7 @@
         <v>50</v>
       </c>
       <c r="H14" s="3" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="I14" s="3" t="s">
         <v>11</v>
@@ -1484,7 +1463,7 @@
         <v>50</v>
       </c>
       <c r="H15" s="3" t="s">
-        <v>28</v>
+        <v>37</v>
       </c>
       <c r="I15" s="3" t="s">
         <v>11</v>
@@ -1537,7 +1516,7 @@
         <v>50</v>
       </c>
       <c r="H16" s="3" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="I16" s="3" t="s">
         <v>11</v>
@@ -1584,13 +1563,13 @@
         <v>40</v>
       </c>
       <c r="F17" s="3" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="G17" s="3" t="s">
-        <v>40</v>
+        <v>50</v>
       </c>
       <c r="H17" s="3" t="s">
-        <v>40</v>
+        <v>26</v>
       </c>
       <c r="I17" s="3" t="s">
         <v>11</v>
@@ -1610,8 +1589,8 @@
       <c r="N17" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="O17" s="4" t="s">
-        <v>15</v>
+      <c r="O17" s="3" t="s">
+        <v>14</v>
       </c>
       <c r="P17" s="3" t="s">
         <v>12</v>
@@ -1637,13 +1616,13 @@
         <v>40</v>
       </c>
       <c r="F18" s="3" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="G18" s="3" t="s">
         <v>40</v>
       </c>
       <c r="H18" s="3" t="s">
-        <v>10</v>
+        <v>40</v>
       </c>
       <c r="I18" s="3" t="s">
         <v>11</v>
@@ -1663,8 +1642,8 @@
       <c r="N18" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="O18" s="3" t="s">
-        <v>14</v>
+      <c r="O18" s="4" t="s">
+        <v>15</v>
       </c>
       <c r="P18" s="3" t="s">
         <v>12</v>
@@ -1678,7 +1657,7 @@
         <v>9</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="C19" s="3" t="s">
         <v>56</v>
@@ -1725,9 +1704,6 @@
       <c r="Q19" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="R19" s="3" t="s">
-        <v>25</v>
-      </c>
     </row>
     <row r="20" spans="1:18" x14ac:dyDescent="0.4">
       <c r="A20" s="7" t="s">
@@ -1746,13 +1722,13 @@
         <v>40</v>
       </c>
       <c r="F20" s="3" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="G20" s="3" t="s">
-        <v>51</v>
+        <v>40</v>
       </c>
       <c r="H20" s="3" t="s">
-        <v>35</v>
+        <v>10</v>
       </c>
       <c r="I20" s="3" t="s">
         <v>11</v>
@@ -1772,8 +1748,8 @@
       <c r="N20" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="O20" s="4" t="s">
-        <v>22</v>
+      <c r="O20" s="3" t="s">
+        <v>14</v>
       </c>
       <c r="P20" s="3" t="s">
         <v>12</v>
@@ -1808,7 +1784,7 @@
         <v>51</v>
       </c>
       <c r="H21" s="3" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="I21" s="3" t="s">
         <v>11</v>
@@ -1864,7 +1840,7 @@
         <v>51</v>
       </c>
       <c r="H22" s="3" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="I22" s="3" t="s">
         <v>11</v>
@@ -1920,7 +1896,7 @@
         <v>51</v>
       </c>
       <c r="H23" s="3" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="I23" s="3" t="s">
         <v>11</v>
@@ -1970,39 +1946,95 @@
         <v>40</v>
       </c>
       <c r="F24" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="G24" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="H24" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="I24" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="J24" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="K24" s="3">
+        <v>10</v>
+      </c>
+      <c r="L24" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="M24" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="N24" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="O24" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="P24" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="Q24" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="R24" s="3" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="25" spans="1:18" x14ac:dyDescent="0.4">
+      <c r="A25" s="7" t="s">
+        <v>9</v>
+      </c>
+      <c r="B25" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="C25" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="D25" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="E25" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="F25" s="3" t="s">
         <v>53</v>
       </c>
-      <c r="G24" s="3" t="s">
-        <v>40</v>
-      </c>
-      <c r="H24" s="3" t="s">
-        <v>40</v>
-      </c>
-      <c r="I24" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="J24" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="K24" s="3">
-        <v>10</v>
-      </c>
-      <c r="L24" s="3" t="s">
-        <v>34</v>
-      </c>
-      <c r="M24" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="N24" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="O24" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="P24" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="Q24" s="3" t="s">
+      <c r="G25" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="H25" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="I25" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="J25" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="K25" s="3">
+        <v>10</v>
+      </c>
+      <c r="L25" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="M25" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="N25" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="O25" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="P25" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="Q25" s="3" t="s">
         <v>15</v>
       </c>
     </row>

</xml_diff>

<commit_message>
hespdiv binned data fully run, plus B_bdnn_rep scripts from cluster
</commit_message>
<xml_diff>
--- a/analyses_log.xlsx
+++ b/analyses_log.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\SimoesLabAdmin\Documents\BDNN_Arielli\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9F39E905-2B73-4FFA-81A1-BF51CC1378AF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{81AB471A-9C16-422E-8C56-95E3DA3DD86F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1543" yWindow="1311" windowWidth="27111" windowHeight="16020" xr2:uid="{2B31D40A-C581-4DA9-854D-6A8F263900C8}"/>
+    <workbookView xWindow="334" yWindow="1671" windowWidth="31997" windowHeight="16020" xr2:uid="{2B31D40A-C581-4DA9-854D-6A8F263900C8}"/>
   </bookViews>
   <sheets>
     <sheet name="table" sheetId="2" r:id="rId1"/>
@@ -115,9 +115,6 @@
     <t>CoVar RJMCMC</t>
   </si>
   <si>
-    <t>Tem Only</t>
-  </si>
-  <si>
     <t>Graphed?</t>
   </si>
   <si>
@@ -224,6 +221,9 @@
   </si>
   <si>
     <t>Compare with 1 Myr BDMCMC, no preds, and CoVar RJMCMC</t>
+  </si>
+  <si>
+    <t>Syn No</t>
   </si>
 </sst>
 </file>
@@ -701,28 +701,28 @@
   <sheetData>
     <row r="1" spans="1:19" s="5" customFormat="1" ht="25.75" x14ac:dyDescent="0.4">
       <c r="A1" s="6" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B1" s="5" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="C1" s="5" t="s">
         <v>0</v>
       </c>
       <c r="D1" s="5" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="E1" s="5" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="F1" s="5" t="s">
         <v>1</v>
       </c>
       <c r="G1" s="5" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="H1" s="5" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="I1" s="5" t="s">
         <v>2</v>
@@ -731,7 +731,7 @@
         <v>3</v>
       </c>
       <c r="K1" s="5" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="L1" s="5" t="s">
         <v>4</v>
@@ -749,10 +749,10 @@
         <v>8</v>
       </c>
       <c r="Q1" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="R1" s="5" t="s">
         <v>23</v>
-      </c>
-      <c r="R1" s="5" t="s">
-        <v>24</v>
       </c>
     </row>
     <row r="2" spans="1:19" s="2" customFormat="1" x14ac:dyDescent="0.4">
@@ -760,22 +760,22 @@
         <v>17</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C2" s="3" t="s">
         <v>17</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="F2" s="3" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="G2" s="3" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="H2" s="3" t="s">
         <v>10</v>
@@ -790,10 +790,10 @@
         <v>10</v>
       </c>
       <c r="L2" s="3" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="M2" s="3" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="N2" s="3" t="s">
         <v>14</v>
@@ -808,7 +808,7 @@
         <v>14</v>
       </c>
       <c r="R2" s="3" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="S2" s="3"/>
     </row>
@@ -817,22 +817,22 @@
         <v>16</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C3" s="3" t="s">
         <v>16</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="F3" s="3" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="G3" s="3" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="H3" s="3" t="s">
         <v>10</v>
@@ -847,10 +847,10 @@
         <v>10</v>
       </c>
       <c r="L3" s="3" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="M3" s="3" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="N3" s="3" t="s">
         <v>14</v>
@@ -865,28 +865,28 @@
         <v>14</v>
       </c>
       <c r="R3" s="3" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="S3" s="2"/>
     </row>
     <row r="4" spans="1:19" s="2" customFormat="1" x14ac:dyDescent="0.4">
       <c r="B4" s="10" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="G4" s="2" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="H4" s="2" t="s">
         <v>10</v>
@@ -901,10 +901,10 @@
         <v>10</v>
       </c>
       <c r="L4" s="3" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="M4" s="2" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="N4" s="2" t="s">
         <v>14</v>
@@ -921,22 +921,22 @@
     </row>
     <row r="5" spans="1:19" s="2" customFormat="1" x14ac:dyDescent="0.4">
       <c r="B5" s="10" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="F5" s="3" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="G5" s="3" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="H5" s="3" t="s">
         <v>10</v>
@@ -951,10 +951,10 @@
         <v>10</v>
       </c>
       <c r="L5" s="3" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="M5" s="3" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="N5" s="2" t="s">
         <v>14</v>
@@ -974,7 +974,7 @@
         <v>21</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C6" s="3" t="s">
         <v>16</v>
@@ -983,16 +983,16 @@
         <v>18</v>
       </c>
       <c r="E6" s="3" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="F6" s="3" t="s">
         <v>20</v>
       </c>
       <c r="G6" s="3" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="H6" s="3" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="I6" s="3" t="s">
         <v>11</v>
@@ -1004,10 +1004,10 @@
         <v>10</v>
       </c>
       <c r="L6" s="3" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="M6" s="3" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="N6" s="3" t="s">
         <v>14</v>
@@ -1027,22 +1027,22 @@
         <v>18</v>
       </c>
       <c r="B7" s="10" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="D7" s="2" t="s">
         <v>18</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="F7" s="2" t="s">
         <v>20</v>
       </c>
       <c r="G7" s="2" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="I7" s="2" t="s">
         <v>11</v>
@@ -1054,10 +1054,10 @@
         <v>10</v>
       </c>
       <c r="L7" s="2" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="M7" s="2" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="N7" s="2" t="s">
         <v>14</v>
@@ -1077,25 +1077,25 @@
         <v>18</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="D8" s="3" t="s">
         <v>18</v>
       </c>
       <c r="E8" s="3" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="F8" s="3" t="s">
         <v>20</v>
       </c>
       <c r="G8" s="3" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="H8" s="3" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="I8" s="3" t="s">
         <v>11</v>
@@ -1107,10 +1107,10 @@
         <v>10</v>
       </c>
       <c r="L8" s="3" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="M8" s="3" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="N8" s="3" t="s">
         <v>14</v>
@@ -1130,25 +1130,25 @@
         <v>19</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C9" s="3" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="D9" s="3" t="s">
         <v>19</v>
       </c>
       <c r="E9" s="3" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="F9" s="3" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="G9" s="3" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="H9" s="3" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="I9" s="3" t="s">
         <v>11</v>
@@ -1160,10 +1160,10 @@
         <v>10</v>
       </c>
       <c r="L9" s="3" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="M9" s="3" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="N9" s="3" t="s">
         <v>14</v>
@@ -1178,7 +1178,7 @@
         <v>14</v>
       </c>
       <c r="R9" s="3" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
     </row>
     <row r="10" spans="1:19" x14ac:dyDescent="0.4">
@@ -1186,25 +1186,25 @@
         <v>19</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C10" s="3" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="D10" s="3" t="s">
         <v>19</v>
       </c>
       <c r="E10" s="3" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="F10" s="3" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="G10" s="3" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="H10" s="3" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="I10" s="3" t="s">
         <v>11</v>
@@ -1216,10 +1216,10 @@
         <v>10</v>
       </c>
       <c r="L10" s="3" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="M10" s="3" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="N10" s="3" t="s">
         <v>14</v>
@@ -1234,7 +1234,7 @@
         <v>15</v>
       </c>
       <c r="R10" s="3" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
     </row>
     <row r="11" spans="1:19" x14ac:dyDescent="0.4">
@@ -1242,25 +1242,25 @@
         <v>19</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C11" s="3" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="D11" s="3" t="s">
         <v>19</v>
       </c>
       <c r="E11" s="3" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="F11" s="3" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="G11" s="3" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="H11" s="3" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="I11" s="3" t="s">
         <v>11</v>
@@ -1272,10 +1272,10 @@
         <v>10</v>
       </c>
       <c r="L11" s="3" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="M11" s="3" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="N11" s="3" t="s">
         <v>14</v>
@@ -1290,7 +1290,7 @@
         <v>15</v>
       </c>
       <c r="R11" s="3" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
     </row>
     <row r="12" spans="1:19" s="8" customFormat="1" x14ac:dyDescent="0.4">
@@ -1298,22 +1298,22 @@
         <v>19</v>
       </c>
       <c r="B12" s="9" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C12" s="8" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="D12" s="8" t="s">
         <v>19</v>
       </c>
       <c r="E12" s="8" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="F12" s="8" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="G12" s="8" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="I12" s="8" t="s">
         <v>11</v>
@@ -1325,10 +1325,10 @@
         <v>10</v>
       </c>
       <c r="L12" s="8" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="M12" s="8" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="N12" s="12" t="s">
         <v>15</v>
@@ -1345,22 +1345,22 @@
         <v>19</v>
       </c>
       <c r="B13" s="9" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C13" s="8" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="D13" s="8" t="s">
         <v>19</v>
       </c>
       <c r="E13" s="8" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="F13" s="8" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="G13" s="8" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="I13" s="8" t="s">
         <v>11</v>
@@ -1372,10 +1372,10 @@
         <v>10</v>
       </c>
       <c r="L13" s="8" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="M13" s="8" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="N13" s="12" t="s">
         <v>15</v>
@@ -1392,25 +1392,25 @@
         <v>9</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C14" s="3" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="D14" s="3" t="s">
         <v>9</v>
       </c>
       <c r="E14" s="3" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="F14" s="3" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="G14" s="3" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="H14" s="3" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="I14" s="3" t="s">
         <v>11</v>
@@ -1422,10 +1422,10 @@
         <v>10</v>
       </c>
       <c r="L14" s="3" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="M14" s="3" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="N14" s="3" t="s">
         <v>14</v>
@@ -1445,25 +1445,25 @@
         <v>9</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C15" s="3" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="D15" s="3" t="s">
         <v>9</v>
       </c>
       <c r="E15" s="3" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="F15" s="3" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="G15" s="3" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="H15" s="3" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="I15" s="3" t="s">
         <v>11</v>
@@ -1475,10 +1475,10 @@
         <v>10</v>
       </c>
       <c r="L15" s="3" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="M15" s="3" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="N15" s="3" t="s">
         <v>14</v>
@@ -1498,25 +1498,25 @@
         <v>9</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C16" s="3" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="D16" s="3" t="s">
         <v>9</v>
       </c>
       <c r="E16" s="3" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="F16" s="3" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="G16" s="3" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="H16" s="3" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="I16" s="3" t="s">
         <v>11</v>
@@ -1528,10 +1528,10 @@
         <v>10</v>
       </c>
       <c r="L16" s="3" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="M16" s="3" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="N16" s="3" t="s">
         <v>14</v>
@@ -1551,25 +1551,25 @@
         <v>9</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C17" s="3" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="D17" s="3" t="s">
         <v>9</v>
       </c>
       <c r="E17" s="3" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="F17" s="3" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="G17" s="3" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="H17" s="3" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="I17" s="3" t="s">
         <v>11</v>
@@ -1581,10 +1581,10 @@
         <v>10</v>
       </c>
       <c r="L17" s="3" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="M17" s="3" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="N17" s="3" t="s">
         <v>14</v>
@@ -1604,25 +1604,25 @@
         <v>9</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C18" s="3" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="D18" s="3" t="s">
         <v>9</v>
       </c>
       <c r="E18" s="3" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="F18" s="3" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="G18" s="3" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="H18" s="3" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="I18" s="3" t="s">
         <v>11</v>
@@ -1634,10 +1634,10 @@
         <v>10</v>
       </c>
       <c r="L18" s="3" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="M18" s="3" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="N18" s="3" t="s">
         <v>14</v>
@@ -1657,22 +1657,22 @@
         <v>9</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C19" s="3" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="D19" s="3" t="s">
         <v>9</v>
       </c>
       <c r="E19" s="3" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="F19" s="3" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="G19" s="3" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="H19" s="3" t="s">
         <v>10</v>
@@ -1687,10 +1687,10 @@
         <v>10</v>
       </c>
       <c r="L19" s="3" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="M19" s="3" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="N19" s="3" t="s">
         <v>14</v>
@@ -1710,22 +1710,22 @@
         <v>9</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C20" s="3" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="D20" s="3" t="s">
         <v>9</v>
       </c>
       <c r="E20" s="3" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="F20" s="3" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="G20" s="3" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="H20" s="3" t="s">
         <v>10</v>
@@ -1740,10 +1740,10 @@
         <v>10</v>
       </c>
       <c r="L20" s="3" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="M20" s="3" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="N20" s="3" t="s">
         <v>14</v>
@@ -1758,7 +1758,7 @@
         <v>15</v>
       </c>
       <c r="R20" s="3" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
     </row>
     <row r="21" spans="1:18" x14ac:dyDescent="0.4">
@@ -1766,25 +1766,25 @@
         <v>9</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C21" s="3" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="D21" s="3" t="s">
         <v>9</v>
       </c>
       <c r="E21" s="3" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="F21" s="3" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="G21" s="3" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="H21" s="3" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="I21" s="3" t="s">
         <v>11</v>
@@ -1796,16 +1796,16 @@
         <v>10</v>
       </c>
       <c r="L21" s="3" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="M21" s="3" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="N21" s="3" t="s">
         <v>14</v>
       </c>
       <c r="O21" s="4" t="s">
-        <v>22</v>
+        <v>58</v>
       </c>
       <c r="P21" s="3" t="s">
         <v>12</v>
@@ -1814,7 +1814,7 @@
         <v>15</v>
       </c>
       <c r="R21" s="3" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
     </row>
     <row r="22" spans="1:18" x14ac:dyDescent="0.4">
@@ -1822,25 +1822,25 @@
         <v>9</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C22" s="3" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="D22" s="3" t="s">
         <v>9</v>
       </c>
       <c r="E22" s="3" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="F22" s="3" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="G22" s="3" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="H22" s="3" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="I22" s="3" t="s">
         <v>11</v>
@@ -1852,16 +1852,16 @@
         <v>10</v>
       </c>
       <c r="L22" s="3" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="M22" s="3" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="N22" s="3" t="s">
         <v>14</v>
       </c>
       <c r="O22" s="4" t="s">
-        <v>22</v>
+        <v>58</v>
       </c>
       <c r="P22" s="3" t="s">
         <v>12</v>
@@ -1870,7 +1870,7 @@
         <v>15</v>
       </c>
       <c r="R22" s="3" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
     </row>
     <row r="23" spans="1:18" x14ac:dyDescent="0.4">
@@ -1878,25 +1878,25 @@
         <v>9</v>
       </c>
       <c r="B23" s="1" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C23" s="3" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="D23" s="3" t="s">
         <v>9</v>
       </c>
       <c r="E23" s="3" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="F23" s="3" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="G23" s="3" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="H23" s="3" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="I23" s="3" t="s">
         <v>11</v>
@@ -1908,16 +1908,16 @@
         <v>10</v>
       </c>
       <c r="L23" s="3" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="M23" s="3" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="N23" s="3" t="s">
         <v>14</v>
       </c>
       <c r="O23" s="4" t="s">
-        <v>22</v>
+        <v>58</v>
       </c>
       <c r="P23" s="3" t="s">
         <v>12</v>
@@ -1926,7 +1926,7 @@
         <v>15</v>
       </c>
       <c r="R23" s="3" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
     </row>
     <row r="24" spans="1:18" x14ac:dyDescent="0.4">
@@ -1934,25 +1934,25 @@
         <v>9</v>
       </c>
       <c r="B24" s="1" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C24" s="3" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="D24" s="3" t="s">
         <v>9</v>
       </c>
       <c r="E24" s="3" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="F24" s="3" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="G24" s="3" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="H24" s="3" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="I24" s="3" t="s">
         <v>11</v>
@@ -1964,16 +1964,16 @@
         <v>10</v>
       </c>
       <c r="L24" s="3" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="M24" s="3" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="N24" s="3" t="s">
         <v>14</v>
       </c>
       <c r="O24" s="4" t="s">
-        <v>22</v>
+        <v>58</v>
       </c>
       <c r="P24" s="3" t="s">
         <v>12</v>
@@ -1982,7 +1982,7 @@
         <v>15</v>
       </c>
       <c r="R24" s="3" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
     </row>
     <row r="25" spans="1:18" x14ac:dyDescent="0.4">
@@ -1990,25 +1990,25 @@
         <v>9</v>
       </c>
       <c r="B25" s="1" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C25" s="3" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="D25" s="3" t="s">
         <v>9</v>
       </c>
       <c r="E25" s="3" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="F25" s="3" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="G25" s="3" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="H25" s="3" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="I25" s="3" t="s">
         <v>11</v>
@@ -2020,10 +2020,10 @@
         <v>10</v>
       </c>
       <c r="L25" s="3" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="M25" s="3" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="N25" s="3" t="s">
         <v>14</v>

</xml_diff>

<commit_message>
renaming files, restoring unfinished B_covar runs, running model probs, general B_covar post processing
</commit_message>
<xml_diff>
--- a/analyses_log.xlsx
+++ b/analyses_log.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\SimoesLabAdmin\Documents\BDNN_Arielli\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8616842C-FEE1-4D76-999A-FF0AD8D9C8DF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C3347825-0F55-4406-98BE-C04515BF432C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="334" yWindow="1671" windowWidth="16372" windowHeight="16020" xr2:uid="{2B31D40A-C581-4DA9-854D-6A8F263900C8}"/>
+    <workbookView xWindow="15334" yWindow="866" windowWidth="16372" windowHeight="16020" xr2:uid="{2B31D40A-C581-4DA9-854D-6A8F263900C8}"/>
   </bookViews>
   <sheets>
     <sheet name="table" sheetId="2" r:id="rId1"/>
@@ -47,7 +47,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="482" uniqueCount="79">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="483" uniqueCount="81">
   <si>
     <t>Sampling Algorithm</t>
   </si>
@@ -259,12 +259,6 @@
     <t>*All Models use a Time Variable Poisson Process (TPP) to model Preservation, except for CoVar RJMCMC HPP, which uses a Homogenous Poisson Process</t>
   </si>
   <si>
-    <t>mcmc_predictors/B_covar_rjmcmc &amp; B_covar_rjmcmc_no_translate</t>
-  </si>
-  <si>
-    <t>mcmc_predictors/B_covar_rjmcmc_hpp</t>
-  </si>
-  <si>
     <t>If 2 directories are indicated (by an "&amp;"), these are the same models w/ one difference in hyperparameter</t>
   </si>
   <si>
@@ -284,6 +278,18 @@
   </si>
   <si>
     <t>mcmc_fixshift_no_predictors/D_bdnn &amp; D_bdnn_update</t>
+  </si>
+  <si>
+    <t>mcmc_fixshift_predictors/D_mcmc</t>
+  </si>
+  <si>
+    <t>mcmc_predictors/B_covar_rjmcmc</t>
+  </si>
+  <si>
+    <t>Good</t>
+  </si>
+  <si>
+    <t>mcmc_predictors/B_covar_rjmcmc_hpp_notranslate</t>
   </si>
 </sst>
 </file>
@@ -923,6 +929,9 @@
       </c>
     </row>
     <row r="4" spans="1:19" x14ac:dyDescent="0.4">
+      <c r="A4" s="3" t="s">
+        <v>77</v>
+      </c>
       <c r="B4" s="3" t="s">
         <v>55</v>
       </c>
@@ -965,8 +974,8 @@
       <c r="O4" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="P4" s="7" t="s">
-        <v>58</v>
+      <c r="P4" s="3" t="s">
+        <v>14</v>
       </c>
       <c r="Q4" s="3" t="s">
         <v>12</v>
@@ -1033,7 +1042,7 @@
     </row>
     <row r="6" spans="1:19" x14ac:dyDescent="0.4">
       <c r="A6" s="3" t="s">
-        <v>70</v>
+        <v>78</v>
       </c>
       <c r="B6" s="3" t="s">
         <v>21</v>
@@ -1081,15 +1090,15 @@
         <v>14</v>
       </c>
       <c r="Q6" s="3" t="s">
-        <v>12</v>
+        <v>79</v>
       </c>
       <c r="R6" s="3" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="7" spans="1:19" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:19" ht="12.45" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A7" s="3" t="s">
-        <v>71</v>
+        <v>80</v>
       </c>
       <c r="B7" s="3" t="s">
         <v>68</v>
@@ -1137,7 +1146,7 @@
         <v>14</v>
       </c>
       <c r="Q7" s="3" t="s">
-        <v>12</v>
+        <v>79</v>
       </c>
       <c r="R7" s="3" t="s">
         <v>14</v>
@@ -1198,7 +1207,7 @@
     </row>
     <row r="9" spans="1:19" x14ac:dyDescent="0.4">
       <c r="A9" s="3" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="B9" s="3" t="s">
         <v>18</v>
@@ -1254,7 +1263,7 @@
     </row>
     <row r="10" spans="1:19" x14ac:dyDescent="0.4">
       <c r="A10" s="3" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="B10" s="3" t="s">
         <v>19</v>
@@ -1313,7 +1322,7 @@
     </row>
     <row r="11" spans="1:19" x14ac:dyDescent="0.4">
       <c r="A11" s="3" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="B11" s="3" t="s">
         <v>19</v>
@@ -1372,7 +1381,7 @@
     </row>
     <row r="12" spans="1:19" x14ac:dyDescent="0.4">
       <c r="A12" s="3" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="B12" s="3" t="s">
         <v>19</v>
@@ -1643,7 +1652,7 @@
     </row>
     <row r="17" spans="1:19" x14ac:dyDescent="0.4">
       <c r="A17" s="3" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="B17" s="1" t="s">
         <v>9</v>
@@ -1699,7 +1708,7 @@
     </row>
     <row r="18" spans="1:19" x14ac:dyDescent="0.4">
       <c r="A18" s="3" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="B18" s="1" t="s">
         <v>9</v>
@@ -1755,7 +1764,7 @@
     </row>
     <row r="19" spans="1:19" x14ac:dyDescent="0.4">
       <c r="A19" s="3" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="B19" s="1" t="s">
         <v>9</v>
@@ -1811,7 +1820,7 @@
     </row>
     <row r="20" spans="1:19" x14ac:dyDescent="0.4">
       <c r="A20" s="3" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="B20" s="1" t="s">
         <v>9</v>
@@ -1920,7 +1929,7 @@
     </row>
     <row r="22" spans="1:19" x14ac:dyDescent="0.4">
       <c r="A22" s="3" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="B22" s="1" t="s">
         <v>9</v>
@@ -2324,7 +2333,7 @@
     </row>
     <row r="30" spans="1:19" ht="102.9" x14ac:dyDescent="0.4">
       <c r="A30" s="2" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="B30" s="8" t="s">
         <v>69</v>

</xml_diff>

<commit_message>
ltt graphs code, adding model probs
</commit_message>
<xml_diff>
--- a/analyses_log.xlsx
+++ b/analyses_log.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\SimoesLabAdmin\Documents\BDNN_Arielli\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{436DF9A6-6D45-4810-97AE-F60E6459EFF2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B6491623-3BE9-4AC1-8082-C3FB503E8E89}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="15334" yWindow="866" windowWidth="16372" windowHeight="16020" xr2:uid="{2B31D40A-C581-4DA9-854D-6A8F263900C8}"/>
   </bookViews>
@@ -47,7 +47,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="483" uniqueCount="81">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="484" uniqueCount="83">
   <si>
     <t>Sampling Algorithm</t>
   </si>
@@ -223,9 +223,6 @@
     <t>Compare with 1 Myr BDMCMC, no preds, and CoVar RJMCMC</t>
   </si>
   <si>
-    <t>Tem Only</t>
-  </si>
-  <si>
     <t>Name in Files</t>
   </si>
   <si>
@@ -290,6 +287,15 @@
   </si>
   <si>
     <t>mcmc_predictors/B_covar_rjmcmc_hpp_notranslate</t>
+  </si>
+  <si>
+    <t>mcmc_predictors/B_covar_mcmc</t>
+  </si>
+  <si>
+    <t>Rep Only</t>
+  </si>
+  <si>
+    <t>Tem and Rep Only</t>
   </si>
 </sst>
 </file>
@@ -753,7 +759,7 @@
   <sheetData>
     <row r="1" spans="1:19" s="9" customFormat="1" ht="25.75" x14ac:dyDescent="0.4">
       <c r="A1" s="9" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="B1" s="9" t="s">
         <v>45</v>
@@ -812,7 +818,7 @@
     </row>
     <row r="2" spans="1:19" x14ac:dyDescent="0.4">
       <c r="A2" s="3" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B2" s="3" t="s">
         <v>17</v>
@@ -871,7 +877,7 @@
     </row>
     <row r="3" spans="1:19" x14ac:dyDescent="0.4">
       <c r="A3" s="3" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="B3" s="3" t="s">
         <v>16</v>
@@ -930,7 +936,7 @@
     </row>
     <row r="4" spans="1:19" x14ac:dyDescent="0.4">
       <c r="A4" s="3" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="B4" s="3" t="s">
         <v>55</v>
@@ -986,7 +992,7 @@
     </row>
     <row r="5" spans="1:19" x14ac:dyDescent="0.4">
       <c r="A5" s="3" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="B5" s="3" t="s">
         <v>55</v>
@@ -1042,7 +1048,7 @@
     </row>
     <row r="6" spans="1:19" x14ac:dyDescent="0.4">
       <c r="A6" s="3" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B6" s="3" t="s">
         <v>21</v>
@@ -1090,7 +1096,7 @@
         <v>14</v>
       </c>
       <c r="Q6" s="3" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="R6" s="3" t="s">
         <v>14</v>
@@ -1098,10 +1104,10 @@
     </row>
     <row r="7" spans="1:19" ht="12.45" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A7" s="3" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="C7" s="2" t="s">
         <v>30</v>
@@ -1146,13 +1152,16 @@
         <v>14</v>
       </c>
       <c r="Q7" s="3" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="R7" s="3" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="8" spans="1:19" x14ac:dyDescent="0.4">
+      <c r="A8" s="3" t="s">
+        <v>80</v>
+      </c>
       <c r="B8" s="3" t="s">
         <v>18</v>
       </c>
@@ -1196,7 +1205,7 @@
         <v>14</v>
       </c>
       <c r="P8" s="7" t="s">
-        <v>15</v>
+        <v>81</v>
       </c>
       <c r="Q8" s="3" t="s">
         <v>12</v>
@@ -1207,7 +1216,7 @@
     </row>
     <row r="9" spans="1:19" x14ac:dyDescent="0.4">
       <c r="A9" s="3" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B9" s="3" t="s">
         <v>18</v>
@@ -1263,7 +1272,7 @@
     </row>
     <row r="10" spans="1:19" x14ac:dyDescent="0.4">
       <c r="A10" s="3" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B10" s="3" t="s">
         <v>19</v>
@@ -1322,7 +1331,7 @@
     </row>
     <row r="11" spans="1:19" x14ac:dyDescent="0.4">
       <c r="A11" s="3" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B11" s="3" t="s">
         <v>19</v>
@@ -1381,7 +1390,7 @@
     </row>
     <row r="12" spans="1:19" x14ac:dyDescent="0.4">
       <c r="A12" s="3" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B12" s="3" t="s">
         <v>19</v>
@@ -1652,7 +1661,7 @@
     </row>
     <row r="17" spans="1:19" x14ac:dyDescent="0.4">
       <c r="A17" s="3" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="B17" s="1" t="s">
         <v>9</v>
@@ -1708,7 +1717,7 @@
     </row>
     <row r="18" spans="1:19" x14ac:dyDescent="0.4">
       <c r="A18" s="3" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="B18" s="1" t="s">
         <v>9</v>
@@ -1764,7 +1773,7 @@
     </row>
     <row r="19" spans="1:19" x14ac:dyDescent="0.4">
       <c r="A19" s="3" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="B19" s="1" t="s">
         <v>9</v>
@@ -1820,7 +1829,7 @@
     </row>
     <row r="20" spans="1:19" x14ac:dyDescent="0.4">
       <c r="A20" s="3" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="B20" s="1" t="s">
         <v>9</v>
@@ -1929,7 +1938,7 @@
     </row>
     <row r="22" spans="1:19" x14ac:dyDescent="0.4">
       <c r="A22" s="3" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B22" s="1" t="s">
         <v>9</v>
@@ -1985,7 +1994,7 @@
     </row>
     <row r="23" spans="1:19" x14ac:dyDescent="0.4">
       <c r="A23" s="3" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B23" s="1" t="s">
         <v>9</v>
@@ -2044,7 +2053,7 @@
     </row>
     <row r="24" spans="1:19" x14ac:dyDescent="0.4">
       <c r="A24" s="3" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="B24" s="1" t="s">
         <v>9</v>
@@ -2089,7 +2098,7 @@
         <v>14</v>
       </c>
       <c r="P24" s="7" t="s">
-        <v>58</v>
+        <v>82</v>
       </c>
       <c r="Q24" s="3" t="s">
         <v>12</v>
@@ -2103,7 +2112,7 @@
     </row>
     <row r="25" spans="1:19" x14ac:dyDescent="0.4">
       <c r="A25" s="3" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B25" s="1" t="s">
         <v>9</v>
@@ -2148,7 +2157,7 @@
         <v>14</v>
       </c>
       <c r="P25" s="7" t="s">
-        <v>58</v>
+        <v>82</v>
       </c>
       <c r="Q25" s="3" t="s">
         <v>12</v>
@@ -2162,7 +2171,7 @@
     </row>
     <row r="26" spans="1:19" x14ac:dyDescent="0.4">
       <c r="A26" s="3" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="B26" s="1" t="s">
         <v>9</v>
@@ -2207,7 +2216,7 @@
         <v>14</v>
       </c>
       <c r="P26" s="7" t="s">
-        <v>58</v>
+        <v>82</v>
       </c>
       <c r="Q26" s="3" t="s">
         <v>12</v>
@@ -2221,7 +2230,7 @@
     </row>
     <row r="27" spans="1:19" x14ac:dyDescent="0.4">
       <c r="A27" s="3" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="B27" s="1" t="s">
         <v>9</v>
@@ -2266,7 +2275,7 @@
         <v>14</v>
       </c>
       <c r="P27" s="7" t="s">
-        <v>58</v>
+        <v>82</v>
       </c>
       <c r="Q27" s="3" t="s">
         <v>12</v>
@@ -2333,10 +2342,10 @@
     </row>
     <row r="30" spans="1:19" ht="102.9" x14ac:dyDescent="0.4">
       <c r="A30" s="2" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="B30" s="8" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
b_covar post processing.  a lot of re-runs, deletions, graphing, restoration, combining logs, etc.
</commit_message>
<xml_diff>
--- a/analyses_log.xlsx
+++ b/analyses_log.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\SimoesLabAdmin\Documents\BDNN_Arielli\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B6491623-3BE9-4AC1-8082-C3FB503E8E89}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{26BEEDC1-3295-4291-BE3E-11E9172F87E6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="15334" yWindow="866" windowWidth="16372" windowHeight="16020" xr2:uid="{2B31D40A-C581-4DA9-854D-6A8F263900C8}"/>
   </bookViews>
@@ -16,7 +16,7 @@
     <sheet name="table" sheetId="2" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">table!$B$1:$T$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">table!$B$1:$B$29</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -47,7 +47,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="484" uniqueCount="83">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="467" uniqueCount="80">
   <si>
     <t>Sampling Algorithm</t>
   </si>
@@ -250,9 +250,6 @@
     <t>mcmc_predictors/B_bdnn_stdscaled_cbrt</t>
   </si>
   <si>
-    <t>CoVar RJMCMC *HPP</t>
-  </si>
-  <si>
     <t>*All Models use a Time Variable Poisson Process (TPP) to model Preservation, except for CoVar RJMCMC HPP, which uses a Homogenous Poisson Process</t>
   </si>
   <si>
@@ -286,13 +283,7 @@
     <t>Good</t>
   </si>
   <si>
-    <t>mcmc_predictors/B_covar_rjmcmc_hpp_notranslate</t>
-  </si>
-  <si>
     <t>mcmc_predictors/B_covar_mcmc</t>
-  </si>
-  <si>
-    <t>Rep Only</t>
   </si>
   <si>
     <t>Tem and Rep Only</t>
@@ -733,7 +724,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A9EA881A-93D2-4F0C-B578-B509C4BBF0BD}">
-  <dimension ref="A1:S30"/>
+  <dimension ref="A1:S29"/>
   <sheetFormatPr defaultRowHeight="12.9" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="1" max="1" width="53.921875" style="3" customWidth="1"/>
@@ -936,7 +927,7 @@
     </row>
     <row r="4" spans="1:19" x14ac:dyDescent="0.4">
       <c r="A4" s="3" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B4" s="3" t="s">
         <v>55</v>
@@ -1048,7 +1039,7 @@
     </row>
     <row r="6" spans="1:19" x14ac:dyDescent="0.4">
       <c r="A6" s="3" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="B6" s="3" t="s">
         <v>21</v>
@@ -1096,24 +1087,24 @@
         <v>14</v>
       </c>
       <c r="Q6" s="3" t="s">
+        <v>77</v>
+      </c>
+      <c r="R6" s="3" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="7" spans="1:19" x14ac:dyDescent="0.4">
+      <c r="A7" s="3" t="s">
         <v>78</v>
       </c>
-      <c r="R6" s="3" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="7" spans="1:19" ht="12.45" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A7" s="3" t="s">
-        <v>79</v>
-      </c>
       <c r="B7" s="3" t="s">
-        <v>67</v>
+        <v>18</v>
       </c>
       <c r="C7" s="2" t="s">
         <v>30</v>
       </c>
       <c r="D7" s="3" t="s">
-        <v>16</v>
+        <v>55</v>
       </c>
       <c r="E7" s="3" t="s">
         <v>18</v>
@@ -1148,25 +1139,25 @@
       <c r="O7" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="P7" s="3" t="s">
-        <v>14</v>
+      <c r="P7" s="7" t="s">
+        <v>79</v>
       </c>
       <c r="Q7" s="3" t="s">
-        <v>78</v>
+        <v>12</v>
       </c>
       <c r="R7" s="3" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="8" spans="1:19" x14ac:dyDescent="0.4">
       <c r="A8" s="3" t="s">
-        <v>80</v>
+        <v>69</v>
       </c>
       <c r="B8" s="3" t="s">
         <v>18</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="D8" s="3" t="s">
         <v>55</v>
@@ -1204,8 +1195,8 @@
       <c r="O8" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="P8" s="7" t="s">
-        <v>81</v>
+      <c r="P8" s="3" t="s">
+        <v>14</v>
       </c>
       <c r="Q8" s="3" t="s">
         <v>12</v>
@@ -1216,10 +1207,10 @@
     </row>
     <row r="9" spans="1:19" x14ac:dyDescent="0.4">
       <c r="A9" s="3" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="C9" s="2" t="s">
         <v>31</v>
@@ -1228,16 +1219,16 @@
         <v>55</v>
       </c>
       <c r="E9" s="3" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="F9" s="3" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="G9" s="3" t="s">
-        <v>20</v>
+        <v>26</v>
       </c>
       <c r="H9" s="3" t="s">
-        <v>39</v>
+        <v>49</v>
       </c>
       <c r="I9" s="3" t="s">
         <v>38</v>
@@ -1267,12 +1258,15 @@
         <v>12</v>
       </c>
       <c r="R9" s="3" t="s">
-        <v>15</v>
+        <v>14</v>
+      </c>
+      <c r="S9" s="3" t="s">
+        <v>28</v>
       </c>
     </row>
     <row r="10" spans="1:19" x14ac:dyDescent="0.4">
       <c r="A10" s="3" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="B10" s="3" t="s">
         <v>19</v>
@@ -1287,7 +1281,7 @@
         <v>19</v>
       </c>
       <c r="F10" s="3" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="G10" s="3" t="s">
         <v>26</v>
@@ -1323,7 +1317,7 @@
         <v>12</v>
       </c>
       <c r="R10" s="3" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="S10" s="3" t="s">
         <v>28</v>
@@ -1331,7 +1325,7 @@
     </row>
     <row r="11" spans="1:19" x14ac:dyDescent="0.4">
       <c r="A11" s="3" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="B11" s="3" t="s">
         <v>19</v>
@@ -1346,7 +1340,7 @@
         <v>19</v>
       </c>
       <c r="F11" s="3" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="G11" s="3" t="s">
         <v>26</v>
@@ -1388,63 +1382,57 @@
         <v>28</v>
       </c>
     </row>
-    <row r="12" spans="1:19" x14ac:dyDescent="0.4">
-      <c r="A12" s="3" t="s">
-        <v>70</v>
-      </c>
-      <c r="B12" s="3" t="s">
+    <row r="12" spans="1:19" s="4" customFormat="1" x14ac:dyDescent="0.4">
+      <c r="B12" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="C12" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="D12" s="3" t="s">
-        <v>55</v>
-      </c>
-      <c r="E12" s="3" t="s">
+      <c r="C12" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="D12" s="4" t="s">
+        <v>55</v>
+      </c>
+      <c r="E12" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="F12" s="3" t="s">
-        <v>42</v>
-      </c>
-      <c r="G12" s="3" t="s">
+      <c r="F12" s="4" t="s">
+        <v>41</v>
+      </c>
+      <c r="G12" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="H12" s="3" t="s">
+      <c r="H12" s="4" t="s">
         <v>49</v>
       </c>
-      <c r="I12" s="3" t="s">
+      <c r="I12" s="4" t="s">
         <v>38</v>
       </c>
-      <c r="J12" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="K12" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="L12" s="3">
-        <v>10</v>
-      </c>
-      <c r="M12" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="N12" s="3" t="s">
-        <v>32</v>
-      </c>
-      <c r="O12" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="P12" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="Q12" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="R12" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="S12" s="3" t="s">
-        <v>28</v>
+      <c r="J12" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="K12" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="L12" s="4">
+        <v>10</v>
+      </c>
+      <c r="M12" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="N12" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="O12" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="P12" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="Q12" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="R12" s="4" t="s">
+        <v>15</v>
       </c>
     </row>
     <row r="13" spans="1:19" s="4" customFormat="1" x14ac:dyDescent="0.4">
@@ -1461,7 +1449,7 @@
         <v>19</v>
       </c>
       <c r="F13" s="4" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="G13" s="4" t="s">
         <v>26</v>
@@ -1514,13 +1502,13 @@
         <v>19</v>
       </c>
       <c r="F14" s="4" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="G14" s="4" t="s">
         <v>26</v>
       </c>
       <c r="H14" s="4" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="I14" s="4" t="s">
         <v>38</v>
@@ -1567,7 +1555,7 @@
         <v>19</v>
       </c>
       <c r="F15" s="4" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="G15" s="4" t="s">
         <v>26</v>
@@ -1606,56 +1594,59 @@
         <v>15</v>
       </c>
     </row>
-    <row r="16" spans="1:19" s="4" customFormat="1" x14ac:dyDescent="0.4">
-      <c r="B16" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="C16" s="5" t="s">
-        <v>30</v>
-      </c>
-      <c r="D16" s="4" t="s">
-        <v>55</v>
-      </c>
-      <c r="E16" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="F16" s="4" t="s">
-        <v>42</v>
-      </c>
-      <c r="G16" s="4" t="s">
-        <v>26</v>
-      </c>
-      <c r="H16" s="4" t="s">
-        <v>50</v>
-      </c>
-      <c r="I16" s="4" t="s">
+    <row r="16" spans="1:19" x14ac:dyDescent="0.4">
+      <c r="A16" s="3" t="s">
+        <v>70</v>
+      </c>
+      <c r="B16" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="C16" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="D16" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="E16" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="F16" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="G16" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="H16" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="I16" s="3" t="s">
         <v>38</v>
       </c>
-      <c r="J16" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="K16" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="L16" s="4">
-        <v>10</v>
-      </c>
-      <c r="M16" s="4" t="s">
-        <v>33</v>
-      </c>
-      <c r="N16" s="4" t="s">
-        <v>32</v>
-      </c>
-      <c r="O16" s="6" t="s">
-        <v>15</v>
-      </c>
-      <c r="P16" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="Q16" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="R16" s="4" t="s">
+      <c r="J16" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="K16" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="L16" s="3">
+        <v>10</v>
+      </c>
+      <c r="M16" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="N16" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="O16" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="P16" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="Q16" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="R16" s="3" t="s">
         <v>15</v>
       </c>
     </row>
@@ -1685,7 +1676,7 @@
         <v>49</v>
       </c>
       <c r="I17" s="3" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="J17" s="3" t="s">
         <v>11</v>
@@ -1741,7 +1732,7 @@
         <v>49</v>
       </c>
       <c r="I18" s="3" t="s">
-        <v>36</v>
+        <v>27</v>
       </c>
       <c r="J18" s="3" t="s">
         <v>11</v>
@@ -1797,7 +1788,7 @@
         <v>49</v>
       </c>
       <c r="I19" s="3" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="J19" s="3" t="s">
         <v>11</v>
@@ -1828,9 +1819,6 @@
       </c>
     </row>
     <row r="20" spans="1:19" x14ac:dyDescent="0.4">
-      <c r="A20" s="3" t="s">
-        <v>74</v>
-      </c>
       <c r="B20" s="1" t="s">
         <v>9</v>
       </c>
@@ -1847,13 +1835,13 @@
         <v>39</v>
       </c>
       <c r="G20" s="3" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="H20" s="3" t="s">
-        <v>49</v>
+        <v>39</v>
       </c>
       <c r="I20" s="3" t="s">
-        <v>25</v>
+        <v>38</v>
       </c>
       <c r="J20" s="3" t="s">
         <v>11</v>
@@ -1873,8 +1861,8 @@
       <c r="O20" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="P20" s="3" t="s">
-        <v>14</v>
+      <c r="P20" s="7" t="s">
+        <v>15</v>
       </c>
       <c r="Q20" s="3" t="s">
         <v>12</v>
@@ -1884,6 +1872,9 @@
       </c>
     </row>
     <row r="21" spans="1:19" x14ac:dyDescent="0.4">
+      <c r="A21" s="3" t="s">
+        <v>74</v>
+      </c>
       <c r="B21" s="1" t="s">
         <v>9</v>
       </c>
@@ -1900,13 +1891,13 @@
         <v>39</v>
       </c>
       <c r="G21" s="3" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="H21" s="3" t="s">
         <v>39</v>
       </c>
       <c r="I21" s="3" t="s">
-        <v>38</v>
+        <v>10</v>
       </c>
       <c r="J21" s="3" t="s">
         <v>11</v>
@@ -1926,8 +1917,8 @@
       <c r="O21" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="P21" s="7" t="s">
-        <v>15</v>
+      <c r="P21" s="3" t="s">
+        <v>14</v>
       </c>
       <c r="Q21" s="3" t="s">
         <v>12</v>
@@ -1938,13 +1929,13 @@
     </row>
     <row r="22" spans="1:19" x14ac:dyDescent="0.4">
       <c r="A22" s="3" t="s">
-        <v>75</v>
+        <v>61</v>
       </c>
       <c r="B22" s="1" t="s">
         <v>9</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="D22" s="3" t="s">
         <v>55</v>
@@ -1991,10 +1982,13 @@
       <c r="R22" s="3" t="s">
         <v>15</v>
       </c>
+      <c r="S22" s="3" t="s">
+        <v>24</v>
+      </c>
     </row>
     <row r="23" spans="1:19" x14ac:dyDescent="0.4">
       <c r="A23" s="3" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="B23" s="1" t="s">
         <v>9</v>
@@ -2012,13 +2006,13 @@
         <v>39</v>
       </c>
       <c r="G23" s="3" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="H23" s="3" t="s">
-        <v>39</v>
+        <v>50</v>
       </c>
       <c r="I23" s="3" t="s">
-        <v>10</v>
+        <v>34</v>
       </c>
       <c r="J23" s="3" t="s">
         <v>11</v>
@@ -2038,8 +2032,8 @@
       <c r="O23" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="P23" s="3" t="s">
-        <v>14</v>
+      <c r="P23" s="7" t="s">
+        <v>79</v>
       </c>
       <c r="Q23" s="3" t="s">
         <v>12</v>
@@ -2053,7 +2047,7 @@
     </row>
     <row r="24" spans="1:19" x14ac:dyDescent="0.4">
       <c r="A24" s="3" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="B24" s="1" t="s">
         <v>9</v>
@@ -2077,7 +2071,7 @@
         <v>50</v>
       </c>
       <c r="I24" s="3" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="J24" s="3" t="s">
         <v>11</v>
@@ -2098,7 +2092,7 @@
         <v>14</v>
       </c>
       <c r="P24" s="7" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
       <c r="Q24" s="3" t="s">
         <v>12</v>
@@ -2112,7 +2106,7 @@
     </row>
     <row r="25" spans="1:19" x14ac:dyDescent="0.4">
       <c r="A25" s="3" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="B25" s="1" t="s">
         <v>9</v>
@@ -2136,7 +2130,7 @@
         <v>50</v>
       </c>
       <c r="I25" s="3" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="J25" s="3" t="s">
         <v>11</v>
@@ -2157,7 +2151,7 @@
         <v>14</v>
       </c>
       <c r="P25" s="7" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
       <c r="Q25" s="3" t="s">
         <v>12</v>
@@ -2171,7 +2165,7 @@
     </row>
     <row r="26" spans="1:19" x14ac:dyDescent="0.4">
       <c r="A26" s="3" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="B26" s="1" t="s">
         <v>9</v>
@@ -2195,7 +2189,7 @@
         <v>50</v>
       </c>
       <c r="I26" s="3" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="J26" s="3" t="s">
         <v>11</v>
@@ -2216,7 +2210,7 @@
         <v>14</v>
       </c>
       <c r="P26" s="7" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
       <c r="Q26" s="3" t="s">
         <v>12</v>
@@ -2229,9 +2223,6 @@
       </c>
     </row>
     <row r="27" spans="1:19" x14ac:dyDescent="0.4">
-      <c r="A27" s="3" t="s">
-        <v>66</v>
-      </c>
       <c r="B27" s="1" t="s">
         <v>9</v>
       </c>
@@ -2248,13 +2239,13 @@
         <v>39</v>
       </c>
       <c r="G27" s="3" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="H27" s="3" t="s">
-        <v>50</v>
+        <v>39</v>
       </c>
       <c r="I27" s="3" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="J27" s="3" t="s">
         <v>11</v>
@@ -2275,7 +2266,7 @@
         <v>14</v>
       </c>
       <c r="P27" s="7" t="s">
-        <v>82</v>
+        <v>15</v>
       </c>
       <c r="Q27" s="3" t="s">
         <v>12</v>
@@ -2283,77 +2274,17 @@
       <c r="R27" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="S27" s="3" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="28" spans="1:19" x14ac:dyDescent="0.4">
-      <c r="B28" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="C28" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="D28" s="3" t="s">
-        <v>55</v>
-      </c>
-      <c r="E28" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="F28" s="3" t="s">
-        <v>39</v>
-      </c>
-      <c r="G28" s="3" t="s">
-        <v>52</v>
-      </c>
-      <c r="H28" s="3" t="s">
-        <v>39</v>
-      </c>
-      <c r="I28" s="3" t="s">
-        <v>38</v>
-      </c>
-      <c r="J28" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="K28" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="L28" s="3">
-        <v>10</v>
-      </c>
-      <c r="M28" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="N28" s="3" t="s">
-        <v>32</v>
-      </c>
-      <c r="O28" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="P28" s="7" t="s">
-        <v>15</v>
-      </c>
-      <c r="Q28" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="R28" s="3" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="30" spans="1:19" ht="102.9" x14ac:dyDescent="0.4">
-      <c r="A30" s="2" t="s">
-        <v>69</v>
-      </c>
-      <c r="B30" s="8" t="s">
+    </row>
+    <row r="29" spans="1:19" ht="102.9" x14ac:dyDescent="0.4">
+      <c r="A29" s="2" t="s">
         <v>68</v>
       </c>
+      <c r="B29" s="8" t="s">
+        <v>67</v>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="B1:T1" xr:uid="{A9EA881A-93D2-4F0C-B578-B509C4BBF0BD}">
-    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="B2:T22">
-      <sortCondition descending="1" ref="B1"/>
-    </sortState>
-  </autoFilter>
+  <autoFilter ref="B1:B29" xr:uid="{A9EA881A-93D2-4F0C-B578-B509C4BBF0BD}"/>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="1200" verticalDpi="1200" r:id="rId1"/>

</xml_diff>

<commit_message>
MBD runs, LTT graphs, making sure things are complete and restoring if needed
</commit_message>
<xml_diff>
--- a/analyses_log.xlsx
+++ b/analyses_log.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\SimoesLabAdmin\Documents\BDNN_Arielli\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{26BEEDC1-3295-4291-BE3E-11E9172F87E6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4A6D6307-18BA-44A8-84ED-19C35A4FE7BC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="15334" yWindow="866" windowWidth="16372" windowHeight="16020" xr2:uid="{2B31D40A-C581-4DA9-854D-6A8F263900C8}"/>
   </bookViews>
@@ -47,7 +47,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="467" uniqueCount="80">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="472" uniqueCount="80">
   <si>
     <t>Sampling Algorithm</t>
   </si>
@@ -232,9 +232,6 @@
     <t>mcmc_no_predictors/RJMCMC</t>
   </si>
   <si>
-    <t>mcmc_no_predictors/A_bdnn_update &amp; A_bdnn</t>
-  </si>
-  <si>
     <t>mcmc_no_predictors/A_mcmc</t>
   </si>
   <si>
@@ -250,9 +247,6 @@
     <t>mcmc_predictors/B_bdnn_stdscaled_cbrt</t>
   </si>
   <si>
-    <t>*All Models use a Time Variable Poisson Process (TPP) to model Preservation, except for CoVar RJMCMC HPP, which uses a Homogenous Poisson Process</t>
-  </si>
-  <si>
     <t>If 2 directories are indicated (by an "&amp;"), these are the same models w/ one difference in hyperparameter</t>
   </si>
   <si>
@@ -287,6 +281,12 @@
   </si>
   <si>
     <t>Tem and Rep Only</t>
+  </si>
+  <si>
+    <t>*All Models use a Time Variable Poisson Process (TPP) to model Preservation</t>
+  </si>
+  <si>
+    <t>mcmc_no_predictors/A_bdnn_update &amp; A_bdnn*</t>
   </si>
 </sst>
 </file>
@@ -927,7 +927,7 @@
     </row>
     <row r="4" spans="1:19" x14ac:dyDescent="0.4">
       <c r="A4" s="3" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="B4" s="3" t="s">
         <v>55</v>
@@ -983,7 +983,7 @@
     </row>
     <row r="5" spans="1:19" x14ac:dyDescent="0.4">
       <c r="A5" s="3" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B5" s="3" t="s">
         <v>55</v>
@@ -1039,7 +1039,7 @@
     </row>
     <row r="6" spans="1:19" x14ac:dyDescent="0.4">
       <c r="A6" s="3" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="B6" s="3" t="s">
         <v>21</v>
@@ -1087,7 +1087,7 @@
         <v>14</v>
       </c>
       <c r="Q6" s="3" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="R6" s="3" t="s">
         <v>14</v>
@@ -1095,7 +1095,7 @@
     </row>
     <row r="7" spans="1:19" x14ac:dyDescent="0.4">
       <c r="A7" s="3" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="B7" s="3" t="s">
         <v>18</v>
@@ -1139,19 +1139,22 @@
       <c r="O7" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="P7" s="7" t="s">
-        <v>79</v>
+      <c r="P7" s="3" t="s">
+        <v>14</v>
       </c>
       <c r="Q7" s="3" t="s">
         <v>12</v>
       </c>
       <c r="R7" s="3" t="s">
         <v>15</v>
+      </c>
+      <c r="S7" s="3" t="s">
+        <v>28</v>
       </c>
     </row>
     <row r="8" spans="1:19" x14ac:dyDescent="0.4">
       <c r="A8" s="3" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="B8" s="3" t="s">
         <v>18</v>
@@ -1207,7 +1210,7 @@
     </row>
     <row r="9" spans="1:19" x14ac:dyDescent="0.4">
       <c r="A9" s="3" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="B9" s="3" t="s">
         <v>19</v>
@@ -1266,7 +1269,7 @@
     </row>
     <row r="10" spans="1:19" x14ac:dyDescent="0.4">
       <c r="A10" s="3" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="B10" s="3" t="s">
         <v>19</v>
@@ -1325,7 +1328,7 @@
     </row>
     <row r="11" spans="1:19" x14ac:dyDescent="0.4">
       <c r="A11" s="3" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="B11" s="3" t="s">
         <v>19</v>
@@ -1383,6 +1386,9 @@
       </c>
     </row>
     <row r="12" spans="1:19" s="4" customFormat="1" x14ac:dyDescent="0.4">
+      <c r="A12" s="4" t="s">
+        <v>76</v>
+      </c>
       <c r="B12" s="4" t="s">
         <v>19</v>
       </c>
@@ -1436,6 +1442,9 @@
       </c>
     </row>
     <row r="13" spans="1:19" s="4" customFormat="1" x14ac:dyDescent="0.4">
+      <c r="A13" s="4" t="s">
+        <v>76</v>
+      </c>
       <c r="B13" s="4" t="s">
         <v>19</v>
       </c>
@@ -1489,6 +1498,9 @@
       </c>
     </row>
     <row r="14" spans="1:19" s="4" customFormat="1" x14ac:dyDescent="0.4">
+      <c r="A14" s="4" t="s">
+        <v>76</v>
+      </c>
       <c r="B14" s="4" t="s">
         <v>19</v>
       </c>
@@ -1528,8 +1540,8 @@
       <c r="N14" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="O14" s="6" t="s">
-        <v>15</v>
+      <c r="O14" s="4" t="s">
+        <v>14</v>
       </c>
       <c r="P14" s="4" t="s">
         <v>15</v>
@@ -1542,6 +1554,9 @@
       </c>
     </row>
     <row r="15" spans="1:19" s="4" customFormat="1" x14ac:dyDescent="0.4">
+      <c r="A15" s="4" t="s">
+        <v>76</v>
+      </c>
       <c r="B15" s="4" t="s">
         <v>19</v>
       </c>
@@ -1581,8 +1596,8 @@
       <c r="N15" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="O15" s="6" t="s">
-        <v>15</v>
+      <c r="O15" s="4" t="s">
+        <v>14</v>
       </c>
       <c r="P15" s="4" t="s">
         <v>15</v>
@@ -1596,7 +1611,7 @@
     </row>
     <row r="16" spans="1:19" x14ac:dyDescent="0.4">
       <c r="A16" s="3" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="B16" s="1" t="s">
         <v>9</v>
@@ -1652,7 +1667,7 @@
     </row>
     <row r="17" spans="1:19" x14ac:dyDescent="0.4">
       <c r="A17" s="3" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="B17" s="1" t="s">
         <v>9</v>
@@ -1708,7 +1723,7 @@
     </row>
     <row r="18" spans="1:19" x14ac:dyDescent="0.4">
       <c r="A18" s="3" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="B18" s="1" t="s">
         <v>9</v>
@@ -1764,7 +1779,7 @@
     </row>
     <row r="19" spans="1:19" x14ac:dyDescent="0.4">
       <c r="A19" s="3" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="B19" s="1" t="s">
         <v>9</v>
@@ -1873,7 +1888,7 @@
     </row>
     <row r="21" spans="1:19" x14ac:dyDescent="0.4">
       <c r="A21" s="3" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="B21" s="1" t="s">
         <v>9</v>
@@ -1929,7 +1944,7 @@
     </row>
     <row r="22" spans="1:19" x14ac:dyDescent="0.4">
       <c r="A22" s="3" t="s">
-        <v>61</v>
+        <v>79</v>
       </c>
       <c r="B22" s="1" t="s">
         <v>9</v>
@@ -1988,7 +2003,7 @@
     </row>
     <row r="23" spans="1:19" x14ac:dyDescent="0.4">
       <c r="A23" s="3" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="B23" s="1" t="s">
         <v>9</v>
@@ -2033,7 +2048,7 @@
         <v>14</v>
       </c>
       <c r="P23" s="7" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="Q23" s="3" t="s">
         <v>12</v>
@@ -2047,7 +2062,7 @@
     </row>
     <row r="24" spans="1:19" x14ac:dyDescent="0.4">
       <c r="A24" s="3" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="B24" s="1" t="s">
         <v>9</v>
@@ -2092,7 +2107,7 @@
         <v>14</v>
       </c>
       <c r="P24" s="7" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="Q24" s="3" t="s">
         <v>12</v>
@@ -2106,7 +2121,7 @@
     </row>
     <row r="25" spans="1:19" x14ac:dyDescent="0.4">
       <c r="A25" s="3" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B25" s="1" t="s">
         <v>9</v>
@@ -2151,7 +2166,7 @@
         <v>14</v>
       </c>
       <c r="P25" s="7" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="Q25" s="3" t="s">
         <v>12</v>
@@ -2165,7 +2180,7 @@
     </row>
     <row r="26" spans="1:19" x14ac:dyDescent="0.4">
       <c r="A26" s="3" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="B26" s="1" t="s">
         <v>9</v>
@@ -2210,7 +2225,7 @@
         <v>14</v>
       </c>
       <c r="P26" s="7" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="Q26" s="3" t="s">
         <v>12</v>
@@ -2275,12 +2290,12 @@
         <v>15</v>
       </c>
     </row>
-    <row r="29" spans="1:19" ht="102.9" x14ac:dyDescent="0.4">
+    <row r="29" spans="1:19" ht="51.45" x14ac:dyDescent="0.4">
       <c r="A29" s="2" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="B29" s="8" t="s">
-        <v>67</v>
+        <v>78</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
getting unique country codes list + correct bdmcmc run test + rerun of nb + newly labelled occurrences graph
</commit_message>
<xml_diff>
--- a/analyses_log.xlsx
+++ b/analyses_log.xlsx
@@ -8,15 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\SimoesLabAdmin\Documents\BDNN_Arielli\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F997B3A4-5B22-45E9-85B0-8921AB0F2B0A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{93A22EC4-E405-4D4E-A2C5-EBDA91AB8363}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="386" yWindow="1200" windowWidth="20665" windowHeight="16020" xr2:uid="{2B31D40A-C581-4DA9-854D-6A8F263900C8}"/>
+    <workbookView xWindow="-729" yWindow="1569" windowWidth="29263" windowHeight="16020" xr2:uid="{2B31D40A-C581-4DA9-854D-6A8F263900C8}"/>
   </bookViews>
   <sheets>
     <sheet name="table" sheetId="2" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">table!$B$1:$B$29</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">table!$B$1:$B$32</definedName>
     <definedName name="HighlightRow">13</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
@@ -48,7 +48,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="475" uniqueCount="85">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="481" uniqueCount="87">
   <si>
     <t>Sampling Algorithm</t>
   </si>
@@ -293,9 +293,6 @@
     <t>mcmc_predictors/B_bdnn_lats_only</t>
   </si>
   <si>
-    <t>Varies</t>
-  </si>
-  <si>
     <t>Tem reps 4, 7, 9 poor diagnostics</t>
   </si>
   <si>
@@ -303,6 +300,15 @@
   </si>
   <si>
     <t>Diagnostics varied by replicate</t>
+  </si>
+  <si>
+    <t>200 mi</t>
+  </si>
+  <si>
+    <t>Poor</t>
+  </si>
+  <si>
+    <t>MCMC + TI</t>
   </si>
 </sst>
 </file>
@@ -339,12 +345,18 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -359,19 +371,25 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -743,7 +761,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A9EA881A-93D2-4F0C-B578-B509C4BBF0BD}">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="A1:S29"/>
+  <dimension ref="A1:S32"/>
   <sheetFormatPr defaultRowHeight="12.9" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="1" max="1" width="53.921875" style="1" customWidth="1"/>
@@ -826,77 +844,26 @@
         <v>23</v>
       </c>
     </row>
-    <row r="2" spans="1:19" x14ac:dyDescent="0.4">
-      <c r="A2" s="1" t="s">
+    <row r="2" spans="1:19" s="5" customFormat="1" x14ac:dyDescent="0.4">
+      <c r="B2" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="C2" s="5" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="3" spans="1:19" x14ac:dyDescent="0.4">
+      <c r="A3" s="6" t="s">
         <v>59</v>
       </c>
-      <c r="B2" s="1" t="s">
+      <c r="B3" s="1" t="s">
         <v>17</v>
-      </c>
-      <c r="C2" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="D2" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="E2" s="1" t="s">
-        <v>46</v>
-      </c>
-      <c r="F2" s="1" t="s">
-        <v>39</v>
-      </c>
-      <c r="G2" s="1" t="s">
-        <v>39</v>
-      </c>
-      <c r="H2" s="1" t="s">
-        <v>39</v>
-      </c>
-      <c r="I2" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="J2" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="K2" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="L2" s="1">
-        <v>10</v>
-      </c>
-      <c r="M2" s="1" t="s">
-        <v>33</v>
-      </c>
-      <c r="N2" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="O2" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="P2" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="Q2" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="R2" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="S2" s="1" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="3" spans="1:19" x14ac:dyDescent="0.4">
-      <c r="A3" s="1" t="s">
-        <v>60</v>
-      </c>
-      <c r="B3" s="1" t="s">
-        <v>16</v>
       </c>
       <c r="C3" s="2" t="s">
         <v>30</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="E3" s="1" t="s">
         <v>46</v>
@@ -935,27 +902,27 @@
         <v>14</v>
       </c>
       <c r="Q3" s="1" t="s">
-        <v>12</v>
+        <v>75</v>
       </c>
       <c r="R3" s="1" t="s">
         <v>15</v>
       </c>
       <c r="S3" s="1" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
     </row>
     <row r="4" spans="1:19" x14ac:dyDescent="0.4">
       <c r="A4" s="1" t="s">
-        <v>73</v>
+        <v>60</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>55</v>
+        <v>16</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>55</v>
+        <v>16</v>
       </c>
       <c r="E4" s="1" t="s">
         <v>46</v>
@@ -982,7 +949,7 @@
         <v>10</v>
       </c>
       <c r="M4" s="1" t="s">
-        <v>33</v>
+        <v>84</v>
       </c>
       <c r="N4" s="1" t="s">
         <v>32</v>
@@ -994,21 +961,24 @@
         <v>14</v>
       </c>
       <c r="Q4" s="1" t="s">
-        <v>12</v>
+        <v>85</v>
       </c>
       <c r="R4" s="1" t="s">
         <v>15</v>
+      </c>
+      <c r="S4" s="1" t="s">
+        <v>57</v>
       </c>
     </row>
     <row r="5" spans="1:19" x14ac:dyDescent="0.4">
       <c r="A5" s="1" t="s">
-        <v>61</v>
+        <v>73</v>
       </c>
       <c r="B5" s="1" t="s">
         <v>55</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="D5" s="1" t="s">
         <v>55</v>
@@ -1046,46 +1016,43 @@
       <c r="O5" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="P5" s="3" t="s">
-        <v>15</v>
+      <c r="P5" s="1" t="s">
+        <v>14</v>
       </c>
       <c r="Q5" s="1" t="s">
-        <v>81</v>
+        <v>12</v>
       </c>
       <c r="R5" s="1" t="s">
         <v>15</v>
-      </c>
-      <c r="S5" s="1" t="s">
-        <v>82</v>
       </c>
     </row>
     <row r="6" spans="1:19" x14ac:dyDescent="0.4">
       <c r="A6" s="1" t="s">
-        <v>74</v>
+        <v>61</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>21</v>
+        <v>55</v>
       </c>
       <c r="C6" s="2" t="s">
         <v>30</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>16</v>
+        <v>55</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>18</v>
+        <v>46</v>
       </c>
       <c r="F6" s="1" t="s">
         <v>39</v>
       </c>
       <c r="G6" s="1" t="s">
-        <v>20</v>
+        <v>39</v>
       </c>
       <c r="H6" s="1" t="s">
         <v>39</v>
       </c>
       <c r="I6" s="1" t="s">
-        <v>38</v>
+        <v>10</v>
       </c>
       <c r="J6" s="1" t="s">
         <v>11</v>
@@ -1105,155 +1072,61 @@
       <c r="O6" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="P6" s="1" t="s">
-        <v>14</v>
+      <c r="P6" s="3" t="s">
+        <v>15</v>
       </c>
       <c r="Q6" s="1" t="s">
-        <v>75</v>
+        <v>82</v>
       </c>
       <c r="R6" s="1" t="s">
-        <v>14</v>
+        <v>15</v>
+      </c>
+      <c r="S6" s="1" t="s">
+        <v>81</v>
       </c>
     </row>
     <row r="7" spans="1:19" x14ac:dyDescent="0.4">
-      <c r="A7" s="1" t="s">
-        <v>76</v>
-      </c>
       <c r="B7" s="1" t="s">
-        <v>18</v>
+        <v>86</v>
       </c>
       <c r="C7" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="P7" s="3"/>
+    </row>
+    <row r="8" spans="1:19" x14ac:dyDescent="0.4">
+      <c r="B8" s="1" t="s">
+        <v>86</v>
+      </c>
+      <c r="C8" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="D7" s="1" t="s">
-        <v>55</v>
-      </c>
-      <c r="E7" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="F7" s="1" t="s">
-        <v>39</v>
-      </c>
-      <c r="G7" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="H7" s="1" t="s">
-        <v>39</v>
-      </c>
-      <c r="I7" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="J7" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="K7" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="L7" s="1">
-        <v>10</v>
-      </c>
-      <c r="M7" s="1" t="s">
-        <v>33</v>
-      </c>
-      <c r="N7" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="O7" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="P7" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="Q7" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="R7" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="S7" s="1" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="8" spans="1:19" x14ac:dyDescent="0.4">
-      <c r="A8" s="1" t="s">
-        <v>67</v>
-      </c>
-      <c r="B8" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="C8" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="D8" s="1" t="s">
-        <v>55</v>
-      </c>
-      <c r="E8" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="F8" s="1" t="s">
-        <v>39</v>
-      </c>
-      <c r="G8" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="H8" s="1" t="s">
-        <v>39</v>
-      </c>
-      <c r="I8" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="J8" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="K8" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="L8" s="1">
-        <v>10</v>
-      </c>
-      <c r="M8" s="1" t="s">
-        <v>33</v>
-      </c>
-      <c r="N8" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="O8" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="P8" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="Q8" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="R8" s="1" t="s">
-        <v>15</v>
-      </c>
+      <c r="P8" s="3"/>
     </row>
     <row r="9" spans="1:19" x14ac:dyDescent="0.4">
       <c r="A9" s="1" t="s">
-        <v>67</v>
+        <v>74</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>55</v>
+        <v>16</v>
       </c>
       <c r="E9" s="1" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="F9" s="1" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="G9" s="1" t="s">
-        <v>26</v>
+        <v>20</v>
       </c>
       <c r="H9" s="1" t="s">
-        <v>49</v>
+        <v>39</v>
       </c>
       <c r="I9" s="1" t="s">
         <v>38</v>
@@ -1280,39 +1153,36 @@
         <v>14</v>
       </c>
       <c r="Q9" s="1" t="s">
-        <v>12</v>
+        <v>75</v>
       </c>
       <c r="R9" s="1" t="s">
         <v>14</v>
-      </c>
-      <c r="S9" s="1" t="s">
-        <v>28</v>
       </c>
     </row>
     <row r="10" spans="1:19" x14ac:dyDescent="0.4">
       <c r="A10" s="1" t="s">
-        <v>67</v>
+        <v>76</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="D10" s="1" t="s">
         <v>55</v>
       </c>
       <c r="E10" s="1" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="F10" s="1" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="G10" s="1" t="s">
-        <v>26</v>
+        <v>20</v>
       </c>
       <c r="H10" s="1" t="s">
-        <v>49</v>
+        <v>39</v>
       </c>
       <c r="I10" s="1" t="s">
         <v>38</v>
@@ -1339,7 +1209,7 @@
         <v>14</v>
       </c>
       <c r="Q10" s="1" t="s">
-        <v>12</v>
+        <v>75</v>
       </c>
       <c r="R10" s="1" t="s">
         <v>15</v>
@@ -1353,7 +1223,7 @@
         <v>67</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C11" s="2" t="s">
         <v>31</v>
@@ -1362,16 +1232,16 @@
         <v>55</v>
       </c>
       <c r="E11" s="1" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="F11" s="1" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="G11" s="1" t="s">
-        <v>26</v>
+        <v>20</v>
       </c>
       <c r="H11" s="1" t="s">
-        <v>49</v>
+        <v>39</v>
       </c>
       <c r="I11" s="1" t="s">
         <v>38</v>
@@ -1403,19 +1273,16 @@
       <c r="R11" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="S11" s="1" t="s">
-        <v>28</v>
-      </c>
     </row>
     <row r="12" spans="1:19" x14ac:dyDescent="0.4">
       <c r="A12" s="1" t="s">
-        <v>76</v>
+        <v>67</v>
       </c>
       <c r="B12" s="1" t="s">
         <v>19</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="D12" s="1" t="s">
         <v>55</v>
@@ -1424,7 +1291,7 @@
         <v>19</v>
       </c>
       <c r="F12" s="1" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="G12" s="1" t="s">
         <v>26</v>
@@ -1453,25 +1320,28 @@
       <c r="O12" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="P12" s="3" t="s">
-        <v>15</v>
+      <c r="P12" s="1" t="s">
+        <v>14</v>
       </c>
       <c r="Q12" s="1" t="s">
         <v>12</v>
       </c>
       <c r="R12" s="1" t="s">
-        <v>15</v>
+        <v>14</v>
+      </c>
+      <c r="S12" s="1" t="s">
+        <v>28</v>
       </c>
     </row>
     <row r="13" spans="1:19" x14ac:dyDescent="0.4">
       <c r="A13" s="1" t="s">
-        <v>76</v>
+        <v>67</v>
       </c>
       <c r="B13" s="1" t="s">
         <v>19</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="D13" s="1" t="s">
         <v>55</v>
@@ -1480,7 +1350,7 @@
         <v>19</v>
       </c>
       <c r="F13" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="G13" s="1" t="s">
         <v>26</v>
@@ -1509,8 +1379,8 @@
       <c r="O13" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="P13" s="3" t="s">
-        <v>15</v>
+      <c r="P13" s="1" t="s">
+        <v>14</v>
       </c>
       <c r="Q13" s="1" t="s">
         <v>12</v>
@@ -1518,16 +1388,19 @@
       <c r="R13" s="1" t="s">
         <v>15</v>
       </c>
+      <c r="S13" s="1" t="s">
+        <v>28</v>
+      </c>
     </row>
     <row r="14" spans="1:19" x14ac:dyDescent="0.4">
       <c r="A14" s="1" t="s">
-        <v>76</v>
+        <v>67</v>
       </c>
       <c r="B14" s="1" t="s">
         <v>19</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="D14" s="1" t="s">
         <v>55</v>
@@ -1536,13 +1409,13 @@
         <v>19</v>
       </c>
       <c r="F14" s="1" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="G14" s="1" t="s">
         <v>26</v>
       </c>
       <c r="H14" s="1" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="I14" s="1" t="s">
         <v>38</v>
@@ -1573,6 +1446,9 @@
       </c>
       <c r="R14" s="1" t="s">
         <v>15</v>
+      </c>
+      <c r="S14" s="1" t="s">
+        <v>28</v>
       </c>
     </row>
     <row r="15" spans="1:19" x14ac:dyDescent="0.4">
@@ -1592,13 +1468,13 @@
         <v>19</v>
       </c>
       <c r="F15" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="G15" s="1" t="s">
         <v>26</v>
       </c>
       <c r="H15" s="1" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="I15" s="1" t="s">
         <v>38</v>
@@ -1621,8 +1497,8 @@
       <c r="O15" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="P15" s="1" t="s">
-        <v>14</v>
+      <c r="P15" s="3" t="s">
+        <v>15</v>
       </c>
       <c r="Q15" s="1" t="s">
         <v>12</v>
@@ -1633,25 +1509,25 @@
     </row>
     <row r="16" spans="1:19" x14ac:dyDescent="0.4">
       <c r="A16" s="1" t="s">
-        <v>68</v>
+        <v>76</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>9</v>
+        <v>19</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="D16" s="1" t="s">
         <v>55</v>
       </c>
       <c r="E16" s="1" t="s">
-        <v>9</v>
+        <v>19</v>
       </c>
       <c r="F16" s="1" t="s">
-        <v>39</v>
+        <v>42</v>
       </c>
       <c r="G16" s="1" t="s">
-        <v>51</v>
+        <v>26</v>
       </c>
       <c r="H16" s="1" t="s">
         <v>49</v>
@@ -1677,8 +1553,8 @@
       <c r="O16" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="P16" s="1" t="s">
-        <v>14</v>
+      <c r="P16" s="3" t="s">
+        <v>15</v>
       </c>
       <c r="Q16" s="1" t="s">
         <v>12</v>
@@ -1689,31 +1565,31 @@
     </row>
     <row r="17" spans="1:19" x14ac:dyDescent="0.4">
       <c r="A17" s="1" t="s">
-        <v>69</v>
+        <v>76</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>9</v>
+        <v>19</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="D17" s="1" t="s">
         <v>55</v>
       </c>
       <c r="E17" s="1" t="s">
-        <v>9</v>
+        <v>19</v>
       </c>
       <c r="F17" s="1" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="G17" s="1" t="s">
-        <v>51</v>
+        <v>26</v>
       </c>
       <c r="H17" s="1" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="I17" s="1" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="J17" s="1" t="s">
         <v>11</v>
@@ -1745,31 +1621,31 @@
     </row>
     <row r="18" spans="1:19" x14ac:dyDescent="0.4">
       <c r="A18" s="1" t="s">
-        <v>70</v>
+        <v>76</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>9</v>
+        <v>19</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="D18" s="1" t="s">
         <v>55</v>
       </c>
       <c r="E18" s="1" t="s">
-        <v>9</v>
+        <v>19</v>
       </c>
       <c r="F18" s="1" t="s">
-        <v>39</v>
+        <v>42</v>
       </c>
       <c r="G18" s="1" t="s">
-        <v>51</v>
+        <v>26</v>
       </c>
       <c r="H18" s="1" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="I18" s="1" t="s">
-        <v>27</v>
+        <v>38</v>
       </c>
       <c r="J18" s="1" t="s">
         <v>11</v>
@@ -1801,7 +1677,7 @@
     </row>
     <row r="19" spans="1:19" x14ac:dyDescent="0.4">
       <c r="A19" s="1" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
       <c r="B19" s="1" t="s">
         <v>9</v>
@@ -1825,7 +1701,7 @@
         <v>49</v>
       </c>
       <c r="I19" s="1" t="s">
-        <v>25</v>
+        <v>38</v>
       </c>
       <c r="J19" s="1" t="s">
         <v>11</v>
@@ -1856,6 +1732,9 @@
       </c>
     </row>
     <row r="20" spans="1:19" x14ac:dyDescent="0.4">
+      <c r="A20" s="1" t="s">
+        <v>69</v>
+      </c>
       <c r="B20" s="1" t="s">
         <v>9</v>
       </c>
@@ -1872,13 +1751,13 @@
         <v>39</v>
       </c>
       <c r="G20" s="1" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="H20" s="1" t="s">
-        <v>39</v>
+        <v>49</v>
       </c>
       <c r="I20" s="1" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="J20" s="1" t="s">
         <v>11</v>
@@ -1898,8 +1777,8 @@
       <c r="O20" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="P20" s="3" t="s">
-        <v>15</v>
+      <c r="P20" s="1" t="s">
+        <v>14</v>
       </c>
       <c r="Q20" s="1" t="s">
         <v>12</v>
@@ -1910,7 +1789,7 @@
     </row>
     <row r="21" spans="1:19" x14ac:dyDescent="0.4">
       <c r="A21" s="1" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="B21" s="1" t="s">
         <v>9</v>
@@ -1928,13 +1807,13 @@
         <v>39</v>
       </c>
       <c r="G21" s="1" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="H21" s="1" t="s">
-        <v>39</v>
+        <v>49</v>
       </c>
       <c r="I21" s="1" t="s">
-        <v>10</v>
+        <v>27</v>
       </c>
       <c r="J21" s="1" t="s">
         <v>11</v>
@@ -1966,13 +1845,13 @@
     </row>
     <row r="22" spans="1:19" x14ac:dyDescent="0.4">
       <c r="A22" s="1" t="s">
-        <v>79</v>
+        <v>71</v>
       </c>
       <c r="B22" s="1" t="s">
         <v>9</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="D22" s="1" t="s">
         <v>55</v>
@@ -1984,13 +1863,13 @@
         <v>39</v>
       </c>
       <c r="G22" s="1" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="H22" s="1" t="s">
-        <v>39</v>
+        <v>49</v>
       </c>
       <c r="I22" s="1" t="s">
-        <v>10</v>
+        <v>25</v>
       </c>
       <c r="J22" s="1" t="s">
         <v>11</v>
@@ -2019,19 +1898,13 @@
       <c r="R22" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="S22" s="1" t="s">
-        <v>24</v>
-      </c>
     </row>
     <row r="23" spans="1:19" x14ac:dyDescent="0.4">
-      <c r="A23" s="1" t="s">
-        <v>62</v>
-      </c>
       <c r="B23" s="1" t="s">
         <v>9</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="D23" s="1" t="s">
         <v>55</v>
@@ -2043,13 +1916,13 @@
         <v>39</v>
       </c>
       <c r="G23" s="1" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="H23" s="1" t="s">
-        <v>50</v>
+        <v>39</v>
       </c>
       <c r="I23" s="1" t="s">
-        <v>34</v>
+        <v>38</v>
       </c>
       <c r="J23" s="1" t="s">
         <v>11</v>
@@ -2070,7 +1943,7 @@
         <v>14</v>
       </c>
       <c r="P23" s="3" t="s">
-        <v>77</v>
+        <v>15</v>
       </c>
       <c r="Q23" s="1" t="s">
         <v>12</v>
@@ -2078,19 +1951,16 @@
       <c r="R23" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="S23" s="1" t="s">
-        <v>24</v>
-      </c>
     </row>
     <row r="24" spans="1:19" x14ac:dyDescent="0.4">
       <c r="A24" s="1" t="s">
-        <v>63</v>
+        <v>72</v>
       </c>
       <c r="B24" s="1" t="s">
         <v>9</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="D24" s="1" t="s">
         <v>55</v>
@@ -2102,13 +1972,13 @@
         <v>39</v>
       </c>
       <c r="G24" s="1" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="H24" s="1" t="s">
-        <v>50</v>
+        <v>39</v>
       </c>
       <c r="I24" s="1" t="s">
-        <v>35</v>
+        <v>10</v>
       </c>
       <c r="J24" s="1" t="s">
         <v>11</v>
@@ -2128,8 +1998,8 @@
       <c r="O24" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="P24" s="3" t="s">
-        <v>77</v>
+      <c r="P24" s="1" t="s">
+        <v>14</v>
       </c>
       <c r="Q24" s="1" t="s">
         <v>12</v>
@@ -2137,13 +2007,10 @@
       <c r="R24" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="S24" s="1" t="s">
-        <v>24</v>
-      </c>
     </row>
     <row r="25" spans="1:19" x14ac:dyDescent="0.4">
       <c r="A25" s="1" t="s">
-        <v>64</v>
+        <v>79</v>
       </c>
       <c r="B25" s="1" t="s">
         <v>9</v>
@@ -2161,13 +2028,13 @@
         <v>39</v>
       </c>
       <c r="G25" s="1" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="H25" s="1" t="s">
-        <v>50</v>
+        <v>39</v>
       </c>
       <c r="I25" s="1" t="s">
-        <v>36</v>
+        <v>10</v>
       </c>
       <c r="J25" s="1" t="s">
         <v>11</v>
@@ -2187,8 +2054,8 @@
       <c r="O25" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="P25" s="3" t="s">
-        <v>77</v>
+      <c r="P25" s="1" t="s">
+        <v>14</v>
       </c>
       <c r="Q25" s="1" t="s">
         <v>12</v>
@@ -2202,7 +2069,7 @@
     </row>
     <row r="26" spans="1:19" x14ac:dyDescent="0.4">
       <c r="A26" s="1" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="B26" s="1" t="s">
         <v>9</v>
@@ -2226,7 +2093,7 @@
         <v>50</v>
       </c>
       <c r="I26" s="1" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="J26" s="1" t="s">
         <v>11</v>
@@ -2261,7 +2128,7 @@
     </row>
     <row r="27" spans="1:19" x14ac:dyDescent="0.4">
       <c r="A27" s="1" t="s">
-        <v>80</v>
+        <v>63</v>
       </c>
       <c r="B27" s="1" t="s">
         <v>9</v>
@@ -2279,13 +2146,13 @@
         <v>39</v>
       </c>
       <c r="G27" s="1" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="H27" s="1" t="s">
-        <v>39</v>
+        <v>50</v>
       </c>
       <c r="I27" s="1" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="J27" s="1" t="s">
         <v>11</v>
@@ -2305,46 +2172,223 @@
       <c r="O27" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="P27" s="1" t="s">
-        <v>14</v>
+      <c r="P27" s="3" t="s">
+        <v>77</v>
       </c>
       <c r="Q27" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="R27" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="S27" s="1" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="28" spans="1:19" x14ac:dyDescent="0.4">
+      <c r="A28" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="B28" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="C28" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="D28" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="E28" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="F28" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="G28" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="H28" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="I28" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="J28" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="K28" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="L28" s="1">
+        <v>10</v>
+      </c>
+      <c r="M28" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="N28" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="O28" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="P28" s="3" t="s">
+        <v>77</v>
+      </c>
+      <c r="Q28" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="R28" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="S28" s="1" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="29" spans="1:19" x14ac:dyDescent="0.4">
+      <c r="A29" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="B29" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="C29" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="D29" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="E29" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="F29" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="G29" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="H29" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="I29" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="J29" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="K29" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="L29" s="1">
+        <v>10</v>
+      </c>
+      <c r="M29" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="N29" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="O29" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="P29" s="3" t="s">
+        <v>77</v>
+      </c>
+      <c r="Q29" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="R29" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="S29" s="1" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="30" spans="1:19" x14ac:dyDescent="0.4">
+      <c r="A30" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="B30" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="C30" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="D30" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="E30" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="F30" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="G30" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="H30" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="I30" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="J30" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="K30" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="L30" s="1">
+        <v>10</v>
+      </c>
+      <c r="M30" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="N30" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="O30" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="P30" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="Q30" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="R30" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="S30" s="1" t="s">
         <v>83</v>
       </c>
-      <c r="R27" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="S27" s="1" t="s">
-        <v>84</v>
-      </c>
-    </row>
-    <row r="29" spans="1:19" ht="51.45" x14ac:dyDescent="0.4">
-      <c r="A29" s="2" t="s">
+    </row>
+    <row r="32" spans="1:19" ht="51.45" x14ac:dyDescent="0.4">
+      <c r="A32" s="2" t="s">
         <v>66</v>
       </c>
-      <c r="B29" s="2" t="s">
+      <c r="B32" s="2" t="s">
         <v>78</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="B1:B29" xr:uid="{A9EA881A-93D2-4F0C-B578-B509C4BBF0BD}"/>
+  <autoFilter ref="B1:B32" xr:uid="{A9EA881A-93D2-4F0C-B578-B509C4BBF0BD}"/>
   <phoneticPr fontId="1" type="noConversion"/>
-  <conditionalFormatting sqref="A4:XFD4">
-    <cfRule type="expression" dxfId="3" priority="4">
-      <formula>ROW()=CELL("row")</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="A1:S29">
-    <cfRule type="expression" dxfId="2" priority="3">
+  <conditionalFormatting sqref="A1:S32">
+    <cfRule type="expression" dxfId="3" priority="3">
       <formula>"row()=cell(""row"")"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A1:XFD1048576">
+    <cfRule type="expression" dxfId="2" priority="1">
+      <formula>ROW(A1)=HighlightRow</formula>
+    </cfRule>
     <cfRule type="expression" dxfId="1" priority="2">
       <formula>"row()=cell(""row"")"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="0" priority="1">
-      <formula>ROW(A1)=HighlightRow</formula>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A5:XFD5">
+    <cfRule type="expression" dxfId="0" priority="4">
+      <formula>ROW()=CELL("row")</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
proper renaming of sub directories, edit of A_mcmc_syn for resub
</commit_message>
<xml_diff>
--- a/analyses_log.xlsx
+++ b/analyses_log.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\SimoesLabAdmin\Documents\BDNN_Arielli\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{93A22EC4-E405-4D4E-A2C5-EBDA91AB8363}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D8D3A203-9F4C-4E44-8346-2F7505C2DF05}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-729" yWindow="1569" windowWidth="29263" windowHeight="16020" xr2:uid="{2B31D40A-C581-4DA9-854D-6A8F263900C8}"/>
+    <workbookView xWindow="3386" yWindow="1843" windowWidth="23700" windowHeight="15986" xr2:uid="{2B31D40A-C581-4DA9-854D-6A8F263900C8}"/>
   </bookViews>
   <sheets>
     <sheet name="table" sheetId="2" r:id="rId1"/>
@@ -48,7 +48,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="481" uniqueCount="87">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="480" uniqueCount="86">
   <si>
     <t>Sampling Algorithm</t>
   </si>
@@ -233,9 +233,6 @@
     <t>mcmc_no_predictors/RJMCMC</t>
   </si>
   <si>
-    <t>mcmc_no_predictors/A_mcmc</t>
-  </si>
-  <si>
     <t>mcmc_predictors/B_bdnn_stdscaled_only</t>
   </si>
   <si>
@@ -293,9 +290,6 @@
     <t>mcmc_predictors/B_bdnn_lats_only</t>
   </si>
   <si>
-    <t>Tem reps 4, 7, 9 poor diagnostics</t>
-  </si>
-  <si>
     <t>Mixed</t>
   </si>
   <si>
@@ -309,6 +303,9 @@
   </si>
   <si>
     <t>MCMC + TI</t>
+  </si>
+  <si>
+    <t>mcmc_no_predictors/A_mcmc_200_iterations</t>
   </si>
 </sst>
 </file>
@@ -902,7 +899,7 @@
         <v>14</v>
       </c>
       <c r="Q3" s="1" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="R3" s="1" t="s">
         <v>15</v>
@@ -949,7 +946,7 @@
         <v>10</v>
       </c>
       <c r="M4" s="1" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="N4" s="1" t="s">
         <v>32</v>
@@ -961,7 +958,7 @@
         <v>14</v>
       </c>
       <c r="Q4" s="1" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="R4" s="1" t="s">
         <v>15</v>
@@ -972,7 +969,7 @@
     </row>
     <row r="5" spans="1:19" x14ac:dyDescent="0.4">
       <c r="A5" s="1" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="B5" s="1" t="s">
         <v>55</v>
@@ -1028,7 +1025,7 @@
     </row>
     <row r="6" spans="1:19" x14ac:dyDescent="0.4">
       <c r="A6" s="1" t="s">
-        <v>61</v>
+        <v>85</v>
       </c>
       <c r="B6" s="1" t="s">
         <v>55</v>
@@ -1064,7 +1061,7 @@
         <v>10</v>
       </c>
       <c r="M6" s="1" t="s">
-        <v>33</v>
+        <v>82</v>
       </c>
       <c r="N6" s="1" t="s">
         <v>32</v>
@@ -1072,22 +1069,19 @@
       <c r="O6" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="P6" s="3" t="s">
-        <v>15</v>
+      <c r="P6" s="1" t="s">
+        <v>14</v>
       </c>
       <c r="Q6" s="1" t="s">
-        <v>82</v>
+        <v>74</v>
       </c>
       <c r="R6" s="1" t="s">
         <v>15</v>
-      </c>
-      <c r="S6" s="1" t="s">
-        <v>81</v>
       </c>
     </row>
     <row r="7" spans="1:19" x14ac:dyDescent="0.4">
       <c r="B7" s="1" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="C7" s="2" t="s">
         <v>31</v>
@@ -1096,7 +1090,7 @@
     </row>
     <row r="8" spans="1:19" x14ac:dyDescent="0.4">
       <c r="B8" s="1" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="C8" s="2" t="s">
         <v>30</v>
@@ -1105,7 +1099,7 @@
     </row>
     <row r="9" spans="1:19" x14ac:dyDescent="0.4">
       <c r="A9" s="1" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="B9" s="1" t="s">
         <v>21</v>
@@ -1153,7 +1147,7 @@
         <v>14</v>
       </c>
       <c r="Q9" s="1" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="R9" s="1" t="s">
         <v>14</v>
@@ -1161,7 +1155,7 @@
     </row>
     <row r="10" spans="1:19" x14ac:dyDescent="0.4">
       <c r="A10" s="1" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B10" s="1" t="s">
         <v>18</v>
@@ -1209,7 +1203,7 @@
         <v>14</v>
       </c>
       <c r="Q10" s="1" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="R10" s="1" t="s">
         <v>15</v>
@@ -1220,7 +1214,7 @@
     </row>
     <row r="11" spans="1:19" x14ac:dyDescent="0.4">
       <c r="A11" s="1" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="B11" s="1" t="s">
         <v>18</v>
@@ -1276,7 +1270,7 @@
     </row>
     <row r="12" spans="1:19" x14ac:dyDescent="0.4">
       <c r="A12" s="1" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="B12" s="1" t="s">
         <v>19</v>
@@ -1335,7 +1329,7 @@
     </row>
     <row r="13" spans="1:19" x14ac:dyDescent="0.4">
       <c r="A13" s="1" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="B13" s="1" t="s">
         <v>19</v>
@@ -1394,7 +1388,7 @@
     </row>
     <row r="14" spans="1:19" x14ac:dyDescent="0.4">
       <c r="A14" s="1" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="B14" s="1" t="s">
         <v>19</v>
@@ -1453,7 +1447,7 @@
     </row>
     <row r="15" spans="1:19" x14ac:dyDescent="0.4">
       <c r="A15" s="1" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B15" s="1" t="s">
         <v>19</v>
@@ -1509,7 +1503,7 @@
     </row>
     <row r="16" spans="1:19" x14ac:dyDescent="0.4">
       <c r="A16" s="1" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B16" s="1" t="s">
         <v>19</v>
@@ -1565,7 +1559,7 @@
     </row>
     <row r="17" spans="1:19" x14ac:dyDescent="0.4">
       <c r="A17" s="1" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B17" s="1" t="s">
         <v>19</v>
@@ -1621,7 +1615,7 @@
     </row>
     <row r="18" spans="1:19" x14ac:dyDescent="0.4">
       <c r="A18" s="1" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B18" s="1" t="s">
         <v>19</v>
@@ -1677,7 +1671,7 @@
     </row>
     <row r="19" spans="1:19" x14ac:dyDescent="0.4">
       <c r="A19" s="1" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="B19" s="1" t="s">
         <v>9</v>
@@ -1733,7 +1727,7 @@
     </row>
     <row r="20" spans="1:19" x14ac:dyDescent="0.4">
       <c r="A20" s="1" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B20" s="1" t="s">
         <v>9</v>
@@ -1789,7 +1783,7 @@
     </row>
     <row r="21" spans="1:19" x14ac:dyDescent="0.4">
       <c r="A21" s="1" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="B21" s="1" t="s">
         <v>9</v>
@@ -1845,7 +1839,7 @@
     </row>
     <row r="22" spans="1:19" x14ac:dyDescent="0.4">
       <c r="A22" s="1" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B22" s="1" t="s">
         <v>9</v>
@@ -1954,7 +1948,7 @@
     </row>
     <row r="24" spans="1:19" x14ac:dyDescent="0.4">
       <c r="A24" s="1" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="B24" s="1" t="s">
         <v>9</v>
@@ -2010,7 +2004,7 @@
     </row>
     <row r="25" spans="1:19" x14ac:dyDescent="0.4">
       <c r="A25" s="1" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="B25" s="1" t="s">
         <v>9</v>
@@ -2069,7 +2063,7 @@
     </row>
     <row r="26" spans="1:19" x14ac:dyDescent="0.4">
       <c r="A26" s="1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B26" s="1" t="s">
         <v>9</v>
@@ -2114,7 +2108,7 @@
         <v>14</v>
       </c>
       <c r="P26" s="3" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="Q26" s="1" t="s">
         <v>12</v>
@@ -2128,7 +2122,7 @@
     </row>
     <row r="27" spans="1:19" x14ac:dyDescent="0.4">
       <c r="A27" s="1" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="B27" s="1" t="s">
         <v>9</v>
@@ -2173,7 +2167,7 @@
         <v>14</v>
       </c>
       <c r="P27" s="3" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="Q27" s="1" t="s">
         <v>12</v>
@@ -2187,7 +2181,7 @@
     </row>
     <row r="28" spans="1:19" x14ac:dyDescent="0.4">
       <c r="A28" s="1" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="B28" s="1" t="s">
         <v>9</v>
@@ -2232,7 +2226,7 @@
         <v>14</v>
       </c>
       <c r="P28" s="3" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="Q28" s="1" t="s">
         <v>12</v>
@@ -2246,7 +2240,7 @@
     </row>
     <row r="29" spans="1:19" x14ac:dyDescent="0.4">
       <c r="A29" s="1" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B29" s="1" t="s">
         <v>9</v>
@@ -2291,7 +2285,7 @@
         <v>14</v>
       </c>
       <c r="P29" s="3" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="Q29" s="1" t="s">
         <v>12</v>
@@ -2305,7 +2299,7 @@
     </row>
     <row r="30" spans="1:19" x14ac:dyDescent="0.4">
       <c r="A30" s="1" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="B30" s="1" t="s">
         <v>9</v>
@@ -2353,21 +2347,21 @@
         <v>14</v>
       </c>
       <c r="Q30" s="1" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="R30" s="1" t="s">
         <v>15</v>
       </c>
       <c r="S30" s="1" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
     </row>
     <row r="32" spans="1:19" ht="51.45" x14ac:dyDescent="0.4">
       <c r="A32" s="2" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="B32" s="2" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
starting mbd runs 1 myr temp C_covar, rerun of eda to output spatial occs graphs by rep, syn, tem, and all taxa age range plot
</commit_message>
<xml_diff>
--- a/analyses_log.xlsx
+++ b/analyses_log.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\SimoesLabAdmin\Documents\BDNN_Arielli\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D8D3A203-9F4C-4E44-8346-2F7505C2DF05}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{65D06806-62AE-437A-ACEB-C4540804353E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3386" yWindow="1843" windowWidth="23700" windowHeight="15986" xr2:uid="{2B31D40A-C581-4DA9-854D-6A8F263900C8}"/>
+    <workbookView xWindow="3386" yWindow="1809" windowWidth="23700" windowHeight="15985" xr2:uid="{2B31D40A-C581-4DA9-854D-6A8F263900C8}"/>
   </bookViews>
   <sheets>
     <sheet name="table" sheetId="2" r:id="rId1"/>
@@ -48,7 +48,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="480" uniqueCount="86">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="528" uniqueCount="86">
   <si>
     <t>Sampling Algorithm</t>
   </si>
@@ -302,10 +302,10 @@
     <t>Poor</t>
   </si>
   <si>
-    <t>MCMC + TI</t>
-  </si>
-  <si>
     <t>mcmc_no_predictors/A_mcmc_200_iterations</t>
+  </si>
+  <si>
+    <t>mcmc_fixshift_no_predictors/BDMCMC</t>
   </si>
 </sst>
 </file>
@@ -368,7 +368,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
@@ -382,17 +382,48 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="4">
+  <dxfs count="8">
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <fill>
         <patternFill>
@@ -841,16 +872,67 @@
         <v>23</v>
       </c>
     </row>
-    <row r="2" spans="1:19" s="5" customFormat="1" x14ac:dyDescent="0.4">
-      <c r="B2" s="5" t="s">
+    <row r="2" spans="1:19" x14ac:dyDescent="0.4">
+      <c r="A2" s="5" t="s">
+        <v>85</v>
+      </c>
+      <c r="B2" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="C2" s="5" t="s">
+      <c r="C2" s="2" t="s">
         <v>31</v>
       </c>
+      <c r="D2" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="F2" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="G2" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="H2" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="I2" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="J2" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="K2" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="L2" s="1">
+        <v>10</v>
+      </c>
+      <c r="M2" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="N2" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="O2" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="P2" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="Q2" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="R2" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="S2" s="1" t="s">
+        <v>56</v>
+      </c>
     </row>
     <row r="3" spans="1:19" x14ac:dyDescent="0.4">
-      <c r="A3" s="6" t="s">
+      <c r="A3" s="5" t="s">
         <v>59</v>
       </c>
       <c r="B3" s="1" t="s">
@@ -895,11 +977,11 @@
       <c r="O3" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="P3" s="1" t="s">
-        <v>14</v>
+      <c r="P3" s="3" t="s">
+        <v>15</v>
       </c>
       <c r="Q3" s="1" t="s">
-        <v>74</v>
+        <v>12</v>
       </c>
       <c r="R3" s="1" t="s">
         <v>15</v>
@@ -1025,7 +1107,7 @@
     </row>
     <row r="6" spans="1:19" x14ac:dyDescent="0.4">
       <c r="A6" s="1" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="B6" s="1" t="s">
         <v>55</v>
@@ -1069,8 +1151,8 @@
       <c r="O6" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="P6" s="1" t="s">
-        <v>14</v>
+      <c r="P6" s="3" t="s">
+        <v>76</v>
       </c>
       <c r="Q6" s="1" t="s">
         <v>74</v>
@@ -1080,35 +1162,132 @@
       </c>
     </row>
     <row r="7" spans="1:19" x14ac:dyDescent="0.4">
+      <c r="A7" s="1" t="s">
+        <v>73</v>
+      </c>
       <c r="B7" s="1" t="s">
-        <v>84</v>
+        <v>21</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="P7" s="3"/>
+        <v>30</v>
+      </c>
+      <c r="D7" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="E7" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="F7" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="G7" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="H7" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="I7" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="J7" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="K7" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="L7" s="1">
+        <v>10</v>
+      </c>
+      <c r="M7" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="N7" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="O7" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="P7" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="Q7" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="R7" s="1" t="s">
+        <v>14</v>
+      </c>
     </row>
     <row r="8" spans="1:19" x14ac:dyDescent="0.4">
+      <c r="A8" s="1" t="s">
+        <v>75</v>
+      </c>
       <c r="B8" s="1" t="s">
-        <v>84</v>
+        <v>18</v>
       </c>
       <c r="C8" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="P8" s="3"/>
+      <c r="D8" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="E8" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="F8" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="G8" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="H8" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="I8" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="J8" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="K8" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="L8" s="1">
+        <v>10</v>
+      </c>
+      <c r="M8" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="N8" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="O8" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="P8" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="Q8" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="R8" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="S8" s="1" t="s">
+        <v>28</v>
+      </c>
     </row>
     <row r="9" spans="1:19" x14ac:dyDescent="0.4">
       <c r="A9" s="1" t="s">
-        <v>73</v>
+        <v>66</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>16</v>
+        <v>55</v>
       </c>
       <c r="E9" s="1" t="s">
         <v>18</v>
@@ -1147,36 +1326,36 @@
         <v>14</v>
       </c>
       <c r="Q9" s="1" t="s">
-        <v>74</v>
+        <v>12</v>
       </c>
       <c r="R9" s="1" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="10" spans="1:19" x14ac:dyDescent="0.4">
       <c r="A10" s="1" t="s">
-        <v>75</v>
+        <v>66</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="D10" s="1" t="s">
         <v>55</v>
       </c>
       <c r="E10" s="1" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="F10" s="1" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="G10" s="1" t="s">
-        <v>20</v>
+        <v>26</v>
       </c>
       <c r="H10" s="1" t="s">
-        <v>39</v>
+        <v>49</v>
       </c>
       <c r="I10" s="1" t="s">
         <v>38</v>
@@ -1203,69 +1382,72 @@
         <v>14</v>
       </c>
       <c r="Q10" s="1" t="s">
-        <v>74</v>
+        <v>12</v>
       </c>
       <c r="R10" s="1" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="S10" s="1" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="11" spans="1:19" x14ac:dyDescent="0.4">
-      <c r="A11" s="1" t="s">
+    <row r="11" spans="1:19" s="6" customFormat="1" x14ac:dyDescent="0.4">
+      <c r="A11" s="6" t="s">
         <v>66</v>
       </c>
-      <c r="B11" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="C11" s="2" t="s">
+      <c r="B11" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="C11" s="7" t="s">
         <v>31</v>
       </c>
-      <c r="D11" s="1" t="s">
-        <v>55</v>
-      </c>
-      <c r="E11" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="F11" s="1" t="s">
-        <v>39</v>
-      </c>
-      <c r="G11" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="H11" s="1" t="s">
-        <v>39</v>
-      </c>
-      <c r="I11" s="1" t="s">
+      <c r="D11" s="6" t="s">
+        <v>55</v>
+      </c>
+      <c r="E11" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="F11" s="6" t="s">
+        <v>41</v>
+      </c>
+      <c r="G11" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="H11" s="6" t="s">
+        <v>49</v>
+      </c>
+      <c r="I11" s="6" t="s">
         <v>38</v>
       </c>
-      <c r="J11" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="K11" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="L11" s="1">
-        <v>10</v>
-      </c>
-      <c r="M11" s="1" t="s">
-        <v>33</v>
-      </c>
-      <c r="N11" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="O11" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="P11" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="Q11" s="1" t="s">
+      <c r="J11" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="K11" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="L11" s="6">
+        <v>10</v>
+      </c>
+      <c r="M11" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="N11" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="O11" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="P11" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="Q11" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="R11" s="1" t="s">
-        <v>15</v>
+      <c r="R11" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="S11" s="6" t="s">
+        <v>28</v>
       </c>
     </row>
     <row r="12" spans="1:19" x14ac:dyDescent="0.4">
@@ -1285,7 +1467,7 @@
         <v>19</v>
       </c>
       <c r="F12" s="1" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="G12" s="1" t="s">
         <v>26</v>
@@ -1321,7 +1503,7 @@
         <v>12</v>
       </c>
       <c r="R12" s="1" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="S12" s="1" t="s">
         <v>28</v>
@@ -1350,7 +1532,7 @@
         <v>26</v>
       </c>
       <c r="H13" s="1" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="I13" s="1" t="s">
         <v>38</v>
@@ -1373,8 +1555,8 @@
       <c r="O13" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="P13" s="1" t="s">
-        <v>14</v>
+      <c r="P13" s="3" t="s">
+        <v>15</v>
       </c>
       <c r="Q13" s="1" t="s">
         <v>12</v>
@@ -1386,7 +1568,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="14" spans="1:19" x14ac:dyDescent="0.4">
+    <row r="14" spans="1:19" ht="12.45" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A14" s="1" t="s">
         <v>66</v>
       </c>
@@ -1409,7 +1591,7 @@
         <v>26</v>
       </c>
       <c r="H14" s="1" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="I14" s="1" t="s">
         <v>38</v>
@@ -1432,8 +1614,8 @@
       <c r="O14" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="P14" s="1" t="s">
-        <v>14</v>
+      <c r="P14" s="3" t="s">
+        <v>15</v>
       </c>
       <c r="Q14" s="1" t="s">
         <v>12</v>
@@ -1491,8 +1673,8 @@
       <c r="O15" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="P15" s="3" t="s">
-        <v>15</v>
+      <c r="P15" s="1" t="s">
+        <v>14</v>
       </c>
       <c r="Q15" s="1" t="s">
         <v>12</v>
@@ -1547,8 +1729,8 @@
       <c r="O16" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="P16" s="3" t="s">
-        <v>15</v>
+      <c r="P16" s="1" t="s">
+        <v>14</v>
       </c>
       <c r="Q16" s="1" t="s">
         <v>12</v>
@@ -2367,24 +2549,6 @@
   </sheetData>
   <autoFilter ref="B1:B32" xr:uid="{A9EA881A-93D2-4F0C-B578-B509C4BBF0BD}"/>
   <phoneticPr fontId="1" type="noConversion"/>
-  <conditionalFormatting sqref="A1:S32">
-    <cfRule type="expression" dxfId="3" priority="3">
-      <formula>"row()=cell(""row"")"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="A1:XFD1048576">
-    <cfRule type="expression" dxfId="2" priority="1">
-      <formula>ROW(A1)=HighlightRow</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="1" priority="2">
-      <formula>"row()=cell(""row"")"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="A5:XFD5">
-    <cfRule type="expression" dxfId="0" priority="4">
-      <formula>ROW()=CELL("row")</formula>
-    </cfRule>
-  </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="1200" verticalDpi="1200" r:id="rId1"/>
 </worksheet>

</xml_diff>